<commit_message>
Las dos hojas de apoyo del panel viajan con sus valores: sus formulas miraban a media plantilla
</commit_message>
<xml_diff>
--- a/panel.xlsx
+++ b/panel.xlsx
@@ -19157,7 +19157,6 @@
         </is>
       </c>
       <c r="C4" s="1345">
-        <f>'PHYSICAL % PROGRESS'!F1</f>
         <v>0</v>
       </c>
     </row>
@@ -19168,7 +19167,6 @@
         </is>
       </c>
       <c r="C5" s="1344" t="str">
-        <f>'PHYSICAL % PROGRESS'!F2</f>
         <v>CONSORCIO CPQ COLUMBITO</v>
       </c>
     </row>
@@ -19179,7 +19177,6 @@
         </is>
       </c>
       <c r="C6" s="1344" t="str">
-        <f>'PHYSICAL % PROGRESS'!F3</f>
         <v>REPOSICION DEL SISTEMA DE FLOCULANTES — LB0</v>
       </c>
     </row>
@@ -19194,224 +19191,170 @@
     <row r="9" spans="2:21" s="1348" customFormat="1">
       <c r="B9" s="1344"/>
       <c r="D9" s="1349">
-        <f>'PHYSICAL % PROGRESS'!P7</f>
         <v>27</v>
       </c>
       <c r="E9" s="1349">
-        <f>'PHYSICAL % PROGRESS'!Q7</f>
         <v>28</v>
       </c>
       <c r="F9" s="1349">
-        <f>'PHYSICAL % PROGRESS'!R7</f>
         <v>29</v>
       </c>
       <c r="G9" s="1349">
-        <f>'PHYSICAL % PROGRESS'!S7</f>
         <v>30</v>
       </c>
       <c r="H9" s="1349">
-        <f>'PHYSICAL % PROGRESS'!T7</f>
         <v>31</v>
       </c>
       <c r="I9" s="1349">
-        <f>'PHYSICAL % PROGRESS'!U7</f>
         <v>32</v>
       </c>
       <c r="J9" s="1349">
-        <f>'PHYSICAL % PROGRESS'!V7</f>
         <v>33</v>
       </c>
       <c r="K9" s="1349">
-        <f>'PHYSICAL % PROGRESS'!W7</f>
         <v>34</v>
       </c>
       <c r="L9" s="1349">
-        <f>'PHYSICAL % PROGRESS'!X7</f>
         <v>35</v>
       </c>
       <c r="M9" s="1349">
-        <f>'PHYSICAL % PROGRESS'!Y7</f>
         <v>36</v>
       </c>
       <c r="N9" s="1349">
-        <f>'PHYSICAL % PROGRESS'!Z7</f>
         <v>37</v>
       </c>
       <c r="O9" s="1349">
-        <f>'PHYSICAL % PROGRESS'!AA7</f>
         <v>38</v>
       </c>
       <c r="P9" s="1349">
-        <f>'PHYSICAL % PROGRESS'!AB7</f>
         <v>39</v>
       </c>
       <c r="Q9" s="1349">
-        <f>'PHYSICAL % PROGRESS'!AC7</f>
         <v>40</v>
       </c>
       <c r="R9" s="1349">
-        <f>'PHYSICAL % PROGRESS'!AD7</f>
         <v>41</v>
       </c>
       <c r="S9" s="1349">
-        <f>'PHYSICAL % PROGRESS'!AE7</f>
         <v>42</v>
       </c>
       <c r="T9" s="1349">
-        <f>'PHYSICAL % PROGRESS'!AF7</f>
         <v>43</v>
       </c>
       <c r="U9" s="1349">
-        <f>'PHYSICAL % PROGRESS'!AG7</f>
         <v>44</v>
       </c>
     </row>
     <row r="10" spans="2:21" s="1348" customFormat="1">
       <c r="B10" s="1344"/>
       <c r="D10" s="1350">
-        <f>'PHYSICAL % PROGRESS'!P8</f>
         <v>46199</v>
       </c>
       <c r="E10" s="1350">
-        <f>'PHYSICAL % PROGRESS'!Q8</f>
         <v>46206</v>
       </c>
       <c r="F10" s="1350">
-        <f>'PHYSICAL % PROGRESS'!R8</f>
         <v>46213</v>
       </c>
       <c r="G10" s="1350">
-        <f>'PHYSICAL % PROGRESS'!S8</f>
         <v>46220</v>
       </c>
       <c r="H10" s="1350">
-        <f>'PHYSICAL % PROGRESS'!T8</f>
         <v>46227</v>
       </c>
       <c r="I10" s="1350">
-        <f>'PHYSICAL % PROGRESS'!U8</f>
         <v>46234</v>
       </c>
       <c r="J10" s="1350">
-        <f>'PHYSICAL % PROGRESS'!V8</f>
         <v>46241</v>
       </c>
       <c r="K10" s="1350">
-        <f>'PHYSICAL % PROGRESS'!W8</f>
         <v>46248</v>
       </c>
       <c r="L10" s="1350">
-        <f>'PHYSICAL % PROGRESS'!X8</f>
         <v>46255</v>
       </c>
       <c r="M10" s="1350">
-        <f>'PHYSICAL % PROGRESS'!Y8</f>
         <v>46262</v>
       </c>
       <c r="N10" s="1350">
-        <f>'PHYSICAL % PROGRESS'!Z8</f>
         <v>46269</v>
       </c>
       <c r="O10" s="1350">
-        <f>'PHYSICAL % PROGRESS'!AA8</f>
         <v>46276</v>
       </c>
       <c r="P10" s="1350">
-        <f>'PHYSICAL % PROGRESS'!AB8</f>
         <v>46283</v>
       </c>
       <c r="Q10" s="1350">
-        <f>'PHYSICAL % PROGRESS'!AC8</f>
         <v>46290</v>
       </c>
       <c r="R10" s="1350">
-        <f>'PHYSICAL % PROGRESS'!AD8</f>
         <v>46297</v>
       </c>
       <c r="S10" s="1350">
-        <f>'PHYSICAL % PROGRESS'!AE8</f>
         <v>46304</v>
       </c>
       <c r="T10" s="1350">
-        <f>'PHYSICAL % PROGRESS'!AF8</f>
         <v>46311</v>
       </c>
       <c r="U10" s="1350">
-        <f>'PHYSICAL % PROGRESS'!AG8</f>
         <v>46318</v>
       </c>
     </row>
     <row r="11" spans="2:21" s="1348" customFormat="1" ht="16.5" thickBot="1">
       <c r="D11" s="1351">
-        <f>'PHYSICAL % PROGRESS'!P9</f>
         <v>46205</v>
       </c>
       <c r="E11" s="1351">
-        <f>'PHYSICAL % PROGRESS'!Q9</f>
         <v>46212</v>
       </c>
       <c r="F11" s="1351">
-        <f>'PHYSICAL % PROGRESS'!R9</f>
         <v>46219</v>
       </c>
       <c r="G11" s="1351">
-        <f>'PHYSICAL % PROGRESS'!S9</f>
         <v>46226</v>
       </c>
       <c r="H11" s="1351">
-        <f>'PHYSICAL % PROGRESS'!T9</f>
         <v>46233</v>
       </c>
       <c r="I11" s="1351">
-        <f>'PHYSICAL % PROGRESS'!U9</f>
         <v>46240</v>
       </c>
       <c r="J11" s="1351">
-        <f>'PHYSICAL % PROGRESS'!V9</f>
         <v>46247</v>
       </c>
       <c r="K11" s="1351">
-        <f>'PHYSICAL % PROGRESS'!W9</f>
         <v>46254</v>
       </c>
       <c r="L11" s="1351">
-        <f>'PHYSICAL % PROGRESS'!X9</f>
         <v>46261</v>
       </c>
       <c r="M11" s="1351">
-        <f>'PHYSICAL % PROGRESS'!Y9</f>
         <v>46268</v>
       </c>
       <c r="N11" s="1351">
-        <f>'PHYSICAL % PROGRESS'!Z9</f>
         <v>46275</v>
       </c>
       <c r="O11" s="1351">
-        <f>'PHYSICAL % PROGRESS'!AA9</f>
         <v>46282</v>
       </c>
       <c r="P11" s="1351">
-        <f>'PHYSICAL % PROGRESS'!AB9</f>
         <v>46289</v>
       </c>
       <c r="Q11" s="1351">
-        <f>'PHYSICAL % PROGRESS'!AC9</f>
         <v>46296</v>
       </c>
       <c r="R11" s="1351">
-        <f>'PHYSICAL % PROGRESS'!AD9</f>
         <v>46303</v>
       </c>
       <c r="S11" s="1351">
-        <f>'PHYSICAL % PROGRESS'!AE9</f>
         <v>46310</v>
       </c>
       <c r="T11" s="1351">
-        <f>'PHYSICAL % PROGRESS'!AF9</f>
         <v>46317</v>
       </c>
       <c r="U11" s="1351">
-        <f>'PHYSICAL % PROGRESS'!AG9</f>
         <v>46324</v>
       </c>
     </row>
@@ -20075,75 +20018,57 @@
         </is>
       </c>
       <c r="D26" s="1364">
-        <f>SUM(D13,D15,D17,D19,D21,D23)</f>
         <v>7</v>
       </c>
       <c r="E26" s="1364">
-        <f t="shared" ref="E26:U26" si="0">SUM(E13,E15,E17,E19,E21,E23)</f>
         <v>7</v>
       </c>
       <c r="F26" s="1364">
-        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="G26" s="1364">
-        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="H26" s="1364">
-        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I26" s="1364">
-        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="J26" s="1364">
-        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="K26" s="1364">
-        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="L26" s="1364">
-        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="M26" s="1364">
-        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="N26" s="1364">
-        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="O26" s="1364">
-        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="P26" s="1364">
-        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="Q26" s="1364">
-        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="R26" s="1364">
-        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="S26" s="1364">
-        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="T26" s="1364">
-        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="U26" s="1364">
-        <f t="shared" si="0"/>
         <v>7</v>
       </c>
     </row>
@@ -20155,75 +20080,57 @@
         </is>
       </c>
       <c r="D27" s="1492">
-        <f>SUM(D14,D16,D18,D20,D22,D24)</f>
         <v>0</v>
       </c>
       <c r="E27" s="1492">
-        <f t="shared" ref="E27:U27" si="1">SUM(E14,E16,E18,E20,E22,E24)</f>
         <v>0</v>
       </c>
       <c r="F27" s="1492">
-        <f>SUM(F14,F16,F18,F20,F22,F24)</f>
         <v>0</v>
       </c>
       <c r="G27" s="1492">
-        <f>SUM(G14,G16,G18,G20,G22,G24)</f>
         <v>8</v>
       </c>
       <c r="H27" s="1492">
-        <f>SUM(H14,H16,H18,H20,H22,H24)</f>
         <v>8</v>
       </c>
       <c r="I27" s="1492">
-        <f>SUM(I14,I16,I18,I20,I22,I24)</f>
         <v>8</v>
       </c>
       <c r="J27" s="1492">
-        <f>SUM(J14,J16,J18,J20,J22,J24)</f>
         <v>8</v>
       </c>
       <c r="K27" s="1492">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="L27" s="1492">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M27" s="1492">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N27" s="1492">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O27" s="1492">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="P27" s="1492">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Q27" s="1492">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R27" s="1492">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="S27" s="1492">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="T27" s="1492">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="U27" s="1492">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -20823,75 +20730,57 @@
         </is>
       </c>
       <c r="D42" s="1364">
-        <f>SUM(D31,D33,D35,D37,D39)</f>
         <v>9</v>
       </c>
       <c r="E42" s="1364">
-        <f t="shared" ref="E42:U42" si="2">SUM(E31,E33,E35,E37,E39)</f>
         <v>9</v>
       </c>
       <c r="F42" s="1364">
-        <f t="shared" si="2"/>
         <v>9</v>
       </c>
       <c r="G42" s="1364">
-        <f t="shared" si="2"/>
         <v>9</v>
       </c>
       <c r="H42" s="1364">
-        <f t="shared" si="2"/>
         <v>9</v>
       </c>
       <c r="I42" s="1364">
-        <f t="shared" si="2"/>
         <v>9</v>
       </c>
       <c r="J42" s="1364">
-        <f t="shared" si="2"/>
         <v>9</v>
       </c>
       <c r="K42" s="1364">
-        <f t="shared" si="2"/>
         <v>9</v>
       </c>
       <c r="L42" s="1364">
-        <f t="shared" si="2"/>
         <v>9</v>
       </c>
       <c r="M42" s="1364">
-        <f t="shared" si="2"/>
         <v>9</v>
       </c>
       <c r="N42" s="1364">
-        <f t="shared" si="2"/>
         <v>9</v>
       </c>
       <c r="O42" s="1364">
-        <f t="shared" si="2"/>
         <v>9</v>
       </c>
       <c r="P42" s="1364">
-        <f t="shared" si="2"/>
         <v>9</v>
       </c>
       <c r="Q42" s="1364">
-        <f t="shared" si="2"/>
         <v>9</v>
       </c>
       <c r="R42" s="1364">
-        <f t="shared" si="2"/>
         <v>9</v>
       </c>
       <c r="S42" s="1364">
-        <f t="shared" si="2"/>
         <v>9</v>
       </c>
       <c r="T42" s="1364">
-        <f t="shared" si="2"/>
         <v>9</v>
       </c>
       <c r="U42" s="1364">
-        <f t="shared" si="2"/>
         <v>9</v>
       </c>
     </row>
@@ -20903,75 +20792,57 @@
         </is>
       </c>
       <c r="D43" s="1492">
-        <f>SUM(D32,D34,D36,D38,D40)</f>
         <v>0</v>
       </c>
       <c r="E43" s="1492">
-        <f t="shared" ref="E43:U43" si="3">SUM(E32,E34,E36,E38,E40)</f>
         <v>0</v>
       </c>
       <c r="F43" s="1492">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="G43" s="1492">
-        <f>SUM(G32,G34,G36,G38,G40)</f>
         <v>5</v>
       </c>
       <c r="H43" s="1492">
-        <f>SUM(H32,H34,H36,H38,H40)</f>
         <v>5</v>
       </c>
       <c r="I43" s="1492">
-        <f>SUM(I32,I34,I36,I38,I40)</f>
         <v>5</v>
       </c>
       <c r="J43" s="1492">
-        <f>SUM(J32,J34,J36,J38,J40)</f>
         <v>5</v>
       </c>
       <c r="K43" s="1492">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L43" s="1492">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="M43" s="1492">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="N43" s="1492">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O43" s="1492">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P43" s="1492">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="Q43" s="1492">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="R43" s="1492">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="S43" s="1492">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="T43" s="1492">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="U43" s="1492">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -21047,7 +20918,6 @@
     </row>
     <row r="47" spans="2:21">
       <c r="B47" s="1499" t="str">
-        <f>'Para Histograma'!D577&amp;"  ("&amp;'Para Histograma'!E577&amp;")"</f>
         <v>CAPATAZ  (CIVIL)</v>
       </c>
       <c r="C47" s="1356" t="inlineStr">
@@ -21056,75 +20926,57 @@
         </is>
       </c>
       <c r="D47" s="1357">
-        <f>'Para Histograma'!L577</f>
         <v>0</v>
       </c>
       <c r="E47" s="1357">
-        <f>'Para Histograma'!M577</f>
         <v>0</v>
       </c>
       <c r="F47" s="1357">
-        <f>'Para Histograma'!N577</f>
         <v>0</v>
       </c>
       <c r="G47" s="1357">
-        <f>'Para Histograma'!O577</f>
         <v>1</v>
       </c>
       <c r="H47" s="1357">
-        <f>'Para Histograma'!P577</f>
         <v>1</v>
       </c>
       <c r="I47" s="1357">
-        <f>'Para Histograma'!Q577</f>
         <v>1</v>
       </c>
       <c r="J47" s="1357">
-        <f>'Para Histograma'!R577</f>
         <v>1</v>
       </c>
       <c r="K47" s="1357">
-        <f>'Para Histograma'!S577</f>
         <v>0</v>
       </c>
       <c r="L47" s="1357">
-        <f>'Para Histograma'!T577</f>
         <v>0</v>
       </c>
       <c r="M47" s="1357">
-        <f>'Para Histograma'!U577</f>
         <v>0</v>
       </c>
       <c r="N47" s="1357">
-        <f>'Para Histograma'!V577</f>
         <v>0</v>
       </c>
       <c r="O47" s="1357">
-        <f>'Para Histograma'!W577</f>
         <v>0</v>
       </c>
       <c r="P47" s="1357">
-        <f>'Para Histograma'!X577</f>
         <v>0</v>
       </c>
       <c r="Q47" s="1357">
-        <f>'Para Histograma'!Y577</f>
         <v>0</v>
       </c>
       <c r="R47" s="1357">
-        <f>'Para Histograma'!Z577</f>
         <v>0</v>
       </c>
       <c r="S47" s="1357">
-        <f>'Para Histograma'!AA577</f>
         <v>0</v>
       </c>
       <c r="T47" s="1357">
-        <f>'Para Histograma'!AB577</f>
         <v>0</v>
       </c>
       <c r="U47" s="1357">
-        <f>'Para Histograma'!AC577</f>
         <v>0</v>
       </c>
     </row>
@@ -21164,7 +21016,6 @@
     </row>
     <row r="49" spans="2:21">
       <c r="B49" s="1499" t="str">
-        <f>'Para Histograma'!D578&amp;"  ("&amp;'Para Histograma'!E578&amp;")"</f>
         <v>AYUDANTE  (CIVIL)</v>
       </c>
       <c r="C49" s="1356" t="inlineStr">
@@ -21173,75 +21024,57 @@
         </is>
       </c>
       <c r="D49" s="1357">
-        <f>'Para Histograma'!L578</f>
         <v>0</v>
       </c>
       <c r="E49" s="1357">
-        <f>'Para Histograma'!M578</f>
         <v>0</v>
       </c>
       <c r="F49" s="1357">
-        <f>'Para Histograma'!N578</f>
         <v>0</v>
       </c>
       <c r="G49" s="1357">
-        <f>'Para Histograma'!O578</f>
         <v>2</v>
       </c>
       <c r="H49" s="1357">
-        <f>'Para Histograma'!P578</f>
         <v>2</v>
       </c>
       <c r="I49" s="1357">
-        <f>'Para Histograma'!Q578</f>
         <v>2</v>
       </c>
       <c r="J49" s="1357">
-        <f>'Para Histograma'!R578</f>
         <v>2</v>
       </c>
       <c r="K49" s="1357">
-        <f>'Para Histograma'!S578</f>
         <v>1</v>
       </c>
       <c r="L49" s="1357">
-        <f>'Para Histograma'!T578</f>
         <v>1</v>
       </c>
       <c r="M49" s="1357">
-        <f>'Para Histograma'!U578</f>
         <v>0</v>
       </c>
       <c r="N49" s="1357">
-        <f>'Para Histograma'!V578</f>
         <v>0</v>
       </c>
       <c r="O49" s="1357">
-        <f>'Para Histograma'!W578</f>
         <v>0</v>
       </c>
       <c r="P49" s="1357">
-        <f>'Para Histograma'!X578</f>
         <v>0</v>
       </c>
       <c r="Q49" s="1357">
-        <f>'Para Histograma'!Y578</f>
         <v>0</v>
       </c>
       <c r="R49" s="1357">
-        <f>'Para Histograma'!Z578</f>
         <v>0</v>
       </c>
       <c r="S49" s="1357">
-        <f>'Para Histograma'!AA578</f>
         <v>0</v>
       </c>
       <c r="T49" s="1357">
-        <f>'Para Histograma'!AB578</f>
         <v>0</v>
       </c>
       <c r="U49" s="1357">
-        <f>'Para Histograma'!AC578</f>
         <v>0</v>
       </c>
     </row>
@@ -21279,7 +21112,6 @@
     </row>
     <row r="51" spans="2:21">
       <c r="B51" s="1499" t="str">
-        <f>'Para Histograma'!D579&amp;"  ("&amp;'Para Histograma'!E579&amp;")"</f>
         <v>OPERARIO  (CIVIL)</v>
       </c>
       <c r="C51" s="1356" t="inlineStr">
@@ -21288,75 +21120,57 @@
         </is>
       </c>
       <c r="D51" s="1357">
-        <f>'Para Histograma'!L579</f>
         <v>0</v>
       </c>
       <c r="E51" s="1357">
-        <f>'Para Histograma'!M579</f>
         <v>0</v>
       </c>
       <c r="F51" s="1357">
-        <f>'Para Histograma'!N579</f>
         <v>0</v>
       </c>
       <c r="G51" s="1357">
-        <f>'Para Histograma'!O579</f>
         <v>0</v>
       </c>
       <c r="H51" s="1357">
-        <f>'Para Histograma'!P579</f>
         <v>1</v>
       </c>
       <c r="I51" s="1357">
-        <f>'Para Histograma'!Q579</f>
         <v>1</v>
       </c>
       <c r="J51" s="1357">
-        <f>'Para Histograma'!R579</f>
         <v>1</v>
       </c>
       <c r="K51" s="1357">
-        <f>'Para Histograma'!S579</f>
         <v>1</v>
       </c>
       <c r="L51" s="1357">
-        <f>'Para Histograma'!T579</f>
         <v>1</v>
       </c>
       <c r="M51" s="1357">
-        <f>'Para Histograma'!U579</f>
         <v>1</v>
       </c>
       <c r="N51" s="1357">
-        <f>'Para Histograma'!V579</f>
         <v>0</v>
       </c>
       <c r="O51" s="1357">
-        <f>'Para Histograma'!W579</f>
         <v>0</v>
       </c>
       <c r="P51" s="1357">
-        <f>'Para Histograma'!X579</f>
         <v>0</v>
       </c>
       <c r="Q51" s="1357">
-        <f>'Para Histograma'!Y579</f>
         <v>0</v>
       </c>
       <c r="R51" s="1357">
-        <f>'Para Histograma'!Z579</f>
         <v>0</v>
       </c>
       <c r="S51" s="1357">
-        <f>'Para Histograma'!AA579</f>
         <v>0</v>
       </c>
       <c r="T51" s="1357">
-        <f>'Para Histograma'!AB579</f>
         <v>0</v>
       </c>
       <c r="U51" s="1357">
-        <f>'Para Histograma'!AC579</f>
         <v>0</v>
       </c>
     </row>
@@ -21388,7 +21202,6 @@
     </row>
     <row r="53" spans="2:21">
       <c r="B53" s="1499" t="str">
-        <f>'Para Histograma'!D580&amp;"  ("&amp;'Para Histograma'!E580&amp;")"</f>
         <v>OFICIAL  (CIVIL)</v>
       </c>
       <c r="C53" s="1356" t="inlineStr">
@@ -21397,75 +21210,57 @@
         </is>
       </c>
       <c r="D53" s="1357">
-        <f>'Para Histograma'!L580</f>
         <v>0</v>
       </c>
       <c r="E53" s="1357">
-        <f>'Para Histograma'!M580</f>
         <v>0</v>
       </c>
       <c r="F53" s="1357">
-        <f>'Para Histograma'!N580</f>
         <v>1</v>
       </c>
       <c r="G53" s="1357">
-        <f>'Para Histograma'!O580</f>
         <v>1</v>
       </c>
       <c r="H53" s="1357">
-        <f>'Para Histograma'!P580</f>
         <v>1</v>
       </c>
       <c r="I53" s="1357">
-        <f>'Para Histograma'!Q580</f>
         <v>1</v>
       </c>
       <c r="J53" s="1357">
-        <f>'Para Histograma'!R580</f>
         <v>0</v>
       </c>
       <c r="K53" s="1357">
-        <f>'Para Histograma'!S580</f>
         <v>0</v>
       </c>
       <c r="L53" s="1357">
-        <f>'Para Histograma'!T580</f>
         <v>0</v>
       </c>
       <c r="M53" s="1357">
-        <f>'Para Histograma'!U580</f>
         <v>0</v>
       </c>
       <c r="N53" s="1357">
-        <f>'Para Histograma'!V580</f>
         <v>0</v>
       </c>
       <c r="O53" s="1357">
-        <f>'Para Histograma'!W580</f>
         <v>0</v>
       </c>
       <c r="P53" s="1357">
-        <f>'Para Histograma'!X580</f>
         <v>0</v>
       </c>
       <c r="Q53" s="1357">
-        <f>'Para Histograma'!Y580</f>
         <v>0</v>
       </c>
       <c r="R53" s="1357">
-        <f>'Para Histograma'!Z580</f>
         <v>0</v>
       </c>
       <c r="S53" s="1357">
-        <f>'Para Histograma'!AA580</f>
         <v>0</v>
       </c>
       <c r="T53" s="1357">
-        <f>'Para Histograma'!AB580</f>
         <v>0</v>
       </c>
       <c r="U53" s="1357">
-        <f>'Para Histograma'!AC580</f>
         <v>0</v>
       </c>
     </row>
@@ -21497,7 +21292,6 @@
     </row>
     <row r="55" spans="2:21">
       <c r="B55" s="1499" t="str">
-        <f>'Para Histograma'!D581&amp;"  ("&amp;'Para Histograma'!E581&amp;")"</f>
         <v>CAPATAZ  (MECÁNICO)</v>
       </c>
       <c r="C55" s="1356" t="inlineStr">
@@ -21506,75 +21300,57 @@
         </is>
       </c>
       <c r="D55" s="1357">
-        <f>'Para Histograma'!L581</f>
         <v>0</v>
       </c>
       <c r="E55" s="1357">
-        <f>'Para Histograma'!M581</f>
         <v>0</v>
       </c>
       <c r="F55" s="1357">
-        <f>'Para Histograma'!N581</f>
         <v>0</v>
       </c>
       <c r="G55" s="1357">
-        <f>'Para Histograma'!O581</f>
         <v>0</v>
       </c>
       <c r="H55" s="1357">
-        <f>'Para Histograma'!P581</f>
         <v>0</v>
       </c>
       <c r="I55" s="1357">
-        <f>'Para Histograma'!Q581</f>
         <v>1</v>
       </c>
       <c r="J55" s="1357">
-        <f>'Para Histograma'!R581</f>
         <v>1</v>
       </c>
       <c r="K55" s="1357">
-        <f>'Para Histograma'!S581</f>
         <v>1</v>
       </c>
       <c r="L55" s="1357">
-        <f>'Para Histograma'!T581</f>
         <v>1</v>
       </c>
       <c r="M55" s="1357">
-        <f>'Para Histograma'!U581</f>
         <v>0</v>
       </c>
       <c r="N55" s="1357">
-        <f>'Para Histograma'!V581</f>
         <v>0</v>
       </c>
       <c r="O55" s="1357">
-        <f>'Para Histograma'!W581</f>
         <v>0</v>
       </c>
       <c r="P55" s="1357">
-        <f>'Para Histograma'!X581</f>
         <v>0</v>
       </c>
       <c r="Q55" s="1357">
-        <f>'Para Histograma'!Y581</f>
         <v>0</v>
       </c>
       <c r="R55" s="1357">
-        <f>'Para Histograma'!Z581</f>
         <v>0</v>
       </c>
       <c r="S55" s="1357">
-        <f>'Para Histograma'!AA581</f>
         <v>0</v>
       </c>
       <c r="T55" s="1357">
-        <f>'Para Histograma'!AB581</f>
         <v>0</v>
       </c>
       <c r="U55" s="1357">
-        <f>'Para Histograma'!AC581</f>
         <v>0</v>
       </c>
     </row>
@@ -21606,7 +21382,6 @@
     </row>
     <row r="57" spans="2:21">
       <c r="B57" s="1499" t="str">
-        <f>'Para Histograma'!D582&amp;"  ("&amp;'Para Histograma'!E582&amp;")"</f>
         <v>OPERARIO  (MECÁNICO)</v>
       </c>
       <c r="C57" s="1356" t="inlineStr">
@@ -21615,75 +21390,57 @@
         </is>
       </c>
       <c r="D57" s="1357">
-        <f>'Para Histograma'!L582</f>
         <v>0</v>
       </c>
       <c r="E57" s="1357">
-        <f>'Para Histograma'!M582</f>
         <v>0</v>
       </c>
       <c r="F57" s="1357">
-        <f>'Para Histograma'!N582</f>
         <v>0</v>
       </c>
       <c r="G57" s="1357">
-        <f>'Para Histograma'!O582</f>
         <v>0</v>
       </c>
       <c r="H57" s="1357">
-        <f>'Para Histograma'!P582</f>
         <v>0</v>
       </c>
       <c r="I57" s="1357">
-        <f>'Para Histograma'!Q582</f>
         <v>1</v>
       </c>
       <c r="J57" s="1357">
-        <f>'Para Histograma'!R582</f>
         <v>1</v>
       </c>
       <c r="K57" s="1357">
-        <f>'Para Histograma'!S582</f>
         <v>1</v>
       </c>
       <c r="L57" s="1357">
-        <f>'Para Histograma'!T582</f>
         <v>3</v>
       </c>
       <c r="M57" s="1357">
-        <f>'Para Histograma'!U582</f>
         <v>3</v>
       </c>
       <c r="N57" s="1357">
-        <f>'Para Histograma'!V582</f>
         <v>3</v>
       </c>
       <c r="O57" s="1357">
-        <f>'Para Histograma'!W582</f>
         <v>4</v>
       </c>
       <c r="P57" s="1357">
-        <f>'Para Histograma'!X582</f>
         <v>4</v>
       </c>
       <c r="Q57" s="1357">
-        <f>'Para Histograma'!Y582</f>
         <v>4</v>
       </c>
       <c r="R57" s="1357">
-        <f>'Para Histograma'!Z582</f>
         <v>4</v>
       </c>
       <c r="S57" s="1357">
-        <f>'Para Histograma'!AA582</f>
         <v>2</v>
       </c>
       <c r="T57" s="1357">
-        <f>'Para Histograma'!AB582</f>
         <v>1</v>
       </c>
       <c r="U57" s="1357">
-        <f>'Para Histograma'!AC582</f>
         <v>0</v>
       </c>
     </row>
@@ -21715,7 +21472,6 @@
     </row>
     <row r="59" spans="2:21">
       <c r="B59" s="1499" t="str">
-        <f>'Para Histograma'!D583&amp;"  ("&amp;'Para Histograma'!E583&amp;")"</f>
         <v>AYUDANTE  (MECÁNICO)</v>
       </c>
       <c r="C59" s="1356" t="inlineStr">
@@ -21724,75 +21480,57 @@
         </is>
       </c>
       <c r="D59" s="1357">
-        <f>'Para Histograma'!L583</f>
         <v>0</v>
       </c>
       <c r="E59" s="1357">
-        <f>'Para Histograma'!M583</f>
         <v>0</v>
       </c>
       <c r="F59" s="1357">
-        <f>'Para Histograma'!N583</f>
         <v>0</v>
       </c>
       <c r="G59" s="1357">
-        <f>'Para Histograma'!O583</f>
         <v>0</v>
       </c>
       <c r="H59" s="1357">
-        <f>'Para Histograma'!P583</f>
         <v>0</v>
       </c>
       <c r="I59" s="1357">
-        <f>'Para Histograma'!Q583</f>
         <v>1</v>
       </c>
       <c r="J59" s="1357">
-        <f>'Para Histograma'!R583</f>
         <v>1</v>
       </c>
       <c r="K59" s="1357">
-        <f>'Para Histograma'!S583</f>
         <v>1</v>
       </c>
       <c r="L59" s="1357">
-        <f>'Para Histograma'!T583</f>
         <v>3</v>
       </c>
       <c r="M59" s="1357">
-        <f>'Para Histograma'!U583</f>
         <v>4</v>
       </c>
       <c r="N59" s="1357">
-        <f>'Para Histograma'!V583</f>
         <v>4</v>
       </c>
       <c r="O59" s="1357">
-        <f>'Para Histograma'!W583</f>
         <v>4</v>
       </c>
       <c r="P59" s="1357">
-        <f>'Para Histograma'!X583</f>
         <v>4</v>
       </c>
       <c r="Q59" s="1357">
-        <f>'Para Histograma'!Y583</f>
         <v>3</v>
       </c>
       <c r="R59" s="1357">
-        <f>'Para Histograma'!Z583</f>
         <v>3</v>
       </c>
       <c r="S59" s="1357">
-        <f>'Para Histograma'!AA583</f>
         <v>2</v>
       </c>
       <c r="T59" s="1357">
-        <f>'Para Histograma'!AB583</f>
         <v>2</v>
       </c>
       <c r="U59" s="1357">
-        <f>'Para Histograma'!AC583</f>
         <v>0</v>
       </c>
     </row>
@@ -21824,7 +21562,6 @@
     </row>
     <row r="61" spans="2:21">
       <c r="B61" s="1499" t="str">
-        <f>'Para Histograma'!D584&amp;"  ("&amp;'Para Histograma'!E584&amp;")"</f>
         <v>SOLDADOR  (MECÁNICO)</v>
       </c>
       <c r="C61" s="1356" t="inlineStr">
@@ -21833,75 +21570,57 @@
         </is>
       </c>
       <c r="D61" s="1357">
-        <f>'Para Histograma'!L584</f>
         <v>0</v>
       </c>
       <c r="E61" s="1357">
-        <f>'Para Histograma'!M584</f>
         <v>0</v>
       </c>
       <c r="F61" s="1357">
-        <f>'Para Histograma'!N584</f>
         <v>0</v>
       </c>
       <c r="G61" s="1357">
-        <f>'Para Histograma'!O584</f>
         <v>0</v>
       </c>
       <c r="H61" s="1357">
-        <f>'Para Histograma'!P584</f>
         <v>0</v>
       </c>
       <c r="I61" s="1357">
-        <f>'Para Histograma'!Q584</f>
         <v>0</v>
       </c>
       <c r="J61" s="1357">
-        <f>'Para Histograma'!R584</f>
         <v>0</v>
       </c>
       <c r="K61" s="1357">
-        <f>'Para Histograma'!S584</f>
         <v>2</v>
       </c>
       <c r="L61" s="1357">
-        <f>'Para Histograma'!T584</f>
         <v>2</v>
       </c>
       <c r="M61" s="1357">
-        <f>'Para Histograma'!U584</f>
         <v>2</v>
       </c>
       <c r="N61" s="1357">
-        <f>'Para Histograma'!V584</f>
         <v>2</v>
       </c>
       <c r="O61" s="1357">
-        <f>'Para Histograma'!W584</f>
         <v>2</v>
       </c>
       <c r="P61" s="1357">
-        <f>'Para Histograma'!X584</f>
         <v>2</v>
       </c>
       <c r="Q61" s="1357">
-        <f>'Para Histograma'!Y584</f>
         <v>2</v>
       </c>
       <c r="R61" s="1357">
-        <f>'Para Histograma'!Z584</f>
         <v>2</v>
       </c>
       <c r="S61" s="1357">
-        <f>'Para Histograma'!AA584</f>
         <v>2</v>
       </c>
       <c r="T61" s="1357">
-        <f>'Para Histograma'!AB584</f>
         <v>0</v>
       </c>
       <c r="U61" s="1357">
-        <f>'Para Histograma'!AC584</f>
         <v>0</v>
       </c>
     </row>
@@ -21933,7 +21652,6 @@
     </row>
     <row r="63" spans="2:21">
       <c r="B63" s="1499" t="str">
-        <f>'Para Histograma'!D585&amp;"  ("&amp;'Para Histograma'!E585&amp;")"</f>
         <v>CAPATAZ  (ELÉCTRICO)</v>
       </c>
       <c r="C63" s="1356" t="inlineStr">
@@ -21942,75 +21660,57 @@
         </is>
       </c>
       <c r="D63" s="1357">
-        <f>'Para Histograma'!L585</f>
         <v>0</v>
       </c>
       <c r="E63" s="1357">
-        <f>'Para Histograma'!M585</f>
         <v>0</v>
       </c>
       <c r="F63" s="1357">
-        <f>'Para Histograma'!N585</f>
         <v>0</v>
       </c>
       <c r="G63" s="1357">
-        <f>'Para Histograma'!O585</f>
         <v>0</v>
       </c>
       <c r="H63" s="1357">
-        <f>'Para Histograma'!P585</f>
         <v>0</v>
       </c>
       <c r="I63" s="1357">
-        <f>'Para Histograma'!Q585</f>
         <v>1</v>
       </c>
       <c r="J63" s="1357">
-        <f>'Para Histograma'!R585</f>
         <v>1</v>
       </c>
       <c r="K63" s="1357">
-        <f>'Para Histograma'!S585</f>
         <v>1</v>
       </c>
       <c r="L63" s="1357">
-        <f>'Para Histograma'!T585</f>
         <v>1</v>
       </c>
       <c r="M63" s="1357">
-        <f>'Para Histograma'!U585</f>
         <v>0</v>
       </c>
       <c r="N63" s="1357">
-        <f>'Para Histograma'!V585</f>
         <v>0</v>
       </c>
       <c r="O63" s="1357">
-        <f>'Para Histograma'!W585</f>
         <v>0</v>
       </c>
       <c r="P63" s="1357">
-        <f>'Para Histograma'!X585</f>
         <v>0</v>
       </c>
       <c r="Q63" s="1357">
-        <f>'Para Histograma'!Y585</f>
         <v>0</v>
       </c>
       <c r="R63" s="1357">
-        <f>'Para Histograma'!Z585</f>
         <v>0</v>
       </c>
       <c r="S63" s="1357">
-        <f>'Para Histograma'!AA585</f>
         <v>0</v>
       </c>
       <c r="T63" s="1357">
-        <f>'Para Histograma'!AB585</f>
         <v>0</v>
       </c>
       <c r="U63" s="1357">
-        <f>'Para Histograma'!AC585</f>
         <v>0</v>
       </c>
     </row>
@@ -22042,7 +21742,6 @@
     </row>
     <row r="65" spans="2:21">
       <c r="B65" s="1499" t="str">
-        <f>'Para Histograma'!D586&amp;"  ("&amp;'Para Histograma'!E586&amp;")"</f>
         <v>OPERARIO  (ELÉCTRICO)</v>
       </c>
       <c r="C65" s="1356" t="inlineStr">
@@ -22051,75 +21750,57 @@
         </is>
       </c>
       <c r="D65" s="1357">
-        <f>'Para Histograma'!L586</f>
         <v>0</v>
       </c>
       <c r="E65" s="1357">
-        <f>'Para Histograma'!M586</f>
         <v>0</v>
       </c>
       <c r="F65" s="1357">
-        <f>'Para Histograma'!N586</f>
         <v>0</v>
       </c>
       <c r="G65" s="1357">
-        <f>'Para Histograma'!O586</f>
         <v>0</v>
       </c>
       <c r="H65" s="1357">
-        <f>'Para Histograma'!P586</f>
         <v>0</v>
       </c>
       <c r="I65" s="1357">
-        <f>'Para Histograma'!Q586</f>
         <v>1</v>
       </c>
       <c r="J65" s="1357">
-        <f>'Para Histograma'!R586</f>
         <v>2</v>
       </c>
       <c r="K65" s="1357">
-        <f>'Para Histograma'!S586</f>
         <v>3</v>
       </c>
       <c r="L65" s="1357">
-        <f>'Para Histograma'!T586</f>
         <v>3</v>
       </c>
       <c r="M65" s="1357">
-        <f>'Para Histograma'!U586</f>
         <v>3</v>
       </c>
       <c r="N65" s="1357">
-        <f>'Para Histograma'!V586</f>
         <v>4</v>
       </c>
       <c r="O65" s="1357">
-        <f>'Para Histograma'!W586</f>
         <v>4</v>
       </c>
       <c r="P65" s="1357">
-        <f>'Para Histograma'!X586</f>
         <v>4</v>
       </c>
       <c r="Q65" s="1357">
-        <f>'Para Histograma'!Y586</f>
         <v>4</v>
       </c>
       <c r="R65" s="1357">
-        <f>'Para Histograma'!Z586</f>
         <v>2</v>
       </c>
       <c r="S65" s="1357">
-        <f>'Para Histograma'!AA586</f>
         <v>2</v>
       </c>
       <c r="T65" s="1357">
-        <f>'Para Histograma'!AB586</f>
         <v>1</v>
       </c>
       <c r="U65" s="1357">
-        <f>'Para Histograma'!AC586</f>
         <v>0</v>
       </c>
     </row>
@@ -22151,7 +21832,6 @@
     </row>
     <row r="67" spans="2:21">
       <c r="B67" s="1499" t="str">
-        <f>'Para Histograma'!D587&amp;"  ("&amp;'Para Histograma'!E587&amp;")"</f>
         <v>AYUDANTE  (ELÉCTRICO)</v>
       </c>
       <c r="C67" s="1356" t="inlineStr">
@@ -22160,75 +21840,57 @@
         </is>
       </c>
       <c r="D67" s="1357">
-        <f>'Para Histograma'!L587</f>
         <v>0</v>
       </c>
       <c r="E67" s="1357">
-        <f>'Para Histograma'!M587</f>
         <v>0</v>
       </c>
       <c r="F67" s="1357">
-        <f>'Para Histograma'!N587</f>
         <v>0</v>
       </c>
       <c r="G67" s="1357">
-        <f>'Para Histograma'!O587</f>
         <v>0</v>
       </c>
       <c r="H67" s="1357">
-        <f>'Para Histograma'!P587</f>
         <v>0</v>
       </c>
       <c r="I67" s="1357">
-        <f>'Para Histograma'!Q587</f>
         <v>1</v>
       </c>
       <c r="J67" s="1357">
-        <f>'Para Histograma'!R587</f>
         <v>2</v>
       </c>
       <c r="K67" s="1357">
-        <f>'Para Histograma'!S587</f>
         <v>2</v>
       </c>
       <c r="L67" s="1357">
-        <f>'Para Histograma'!T587</f>
         <v>2</v>
       </c>
       <c r="M67" s="1357">
-        <f>'Para Histograma'!U587</f>
         <v>3</v>
       </c>
       <c r="N67" s="1357">
-        <f>'Para Histograma'!V587</f>
         <v>5</v>
       </c>
       <c r="O67" s="1357">
-        <f>'Para Histograma'!W587</f>
         <v>5</v>
       </c>
       <c r="P67" s="1357">
-        <f>'Para Histograma'!X587</f>
         <v>5</v>
       </c>
       <c r="Q67" s="1357">
-        <f>'Para Histograma'!Y587</f>
         <v>5</v>
       </c>
       <c r="R67" s="1357">
-        <f>'Para Histograma'!Z587</f>
         <v>1</v>
       </c>
       <c r="S67" s="1357">
-        <f>'Para Histograma'!AA587</f>
         <v>1</v>
       </c>
       <c r="T67" s="1357">
-        <f>'Para Histograma'!AB587</f>
         <v>0</v>
       </c>
       <c r="U67" s="1357">
-        <f>'Para Histograma'!AC587</f>
         <v>0</v>
       </c>
     </row>
@@ -22260,7 +21922,6 @@
     </row>
     <row r="69" spans="2:21">
       <c r="B69" s="1499" t="str">
-        <f>'Para Histograma'!D588&amp;"  ("&amp;'Para Histograma'!E588&amp;")"</f>
         <v>CAPATAZ ELECTRICISTA  (ELÉCTRICO)</v>
       </c>
       <c r="C69" s="1356" t="inlineStr">
@@ -22269,75 +21930,57 @@
         </is>
       </c>
       <c r="D69" s="1357">
-        <f>'Para Histograma'!L588</f>
         <v>0</v>
       </c>
       <c r="E69" s="1357">
-        <f>'Para Histograma'!M588</f>
         <v>0</v>
       </c>
       <c r="F69" s="1357">
-        <f>'Para Histograma'!N588</f>
         <v>0</v>
       </c>
       <c r="G69" s="1357">
-        <f>'Para Histograma'!O588</f>
         <v>0</v>
       </c>
       <c r="H69" s="1357">
-        <f>'Para Histograma'!P588</f>
         <v>0</v>
       </c>
       <c r="I69" s="1357">
-        <f>'Para Histograma'!Q588</f>
         <v>0</v>
       </c>
       <c r="J69" s="1357">
-        <f>'Para Histograma'!R588</f>
         <v>0</v>
       </c>
       <c r="K69" s="1357">
-        <f>'Para Histograma'!S588</f>
         <v>1</v>
       </c>
       <c r="L69" s="1357">
-        <f>'Para Histograma'!T588</f>
         <v>1</v>
       </c>
       <c r="M69" s="1357">
-        <f>'Para Histograma'!U588</f>
         <v>1</v>
       </c>
       <c r="N69" s="1357">
-        <f>'Para Histograma'!V588</f>
         <v>1</v>
       </c>
       <c r="O69" s="1357">
-        <f>'Para Histograma'!W588</f>
         <v>0</v>
       </c>
       <c r="P69" s="1357">
-        <f>'Para Histograma'!X588</f>
         <v>0</v>
       </c>
       <c r="Q69" s="1357">
-        <f>'Para Histograma'!Y588</f>
         <v>0</v>
       </c>
       <c r="R69" s="1357">
-        <f>'Para Histograma'!Z588</f>
         <v>0</v>
       </c>
       <c r="S69" s="1357">
-        <f>'Para Histograma'!AA588</f>
         <v>0</v>
       </c>
       <c r="T69" s="1357">
-        <f>'Para Histograma'!AB588</f>
         <v>0</v>
       </c>
       <c r="U69" s="1357">
-        <f>'Para Histograma'!AC588</f>
         <v>0</v>
       </c>
     </row>
@@ -22369,7 +22012,6 @@
     </row>
     <row r="71" spans="2:21">
       <c r="B71" s="1499" t="str">
-        <f>'Para Histograma'!D589&amp;"  ("&amp;'Para Histograma'!E589&amp;")"</f>
         <v>OPERARIO ELECTRICISTA  (ELÉCTRICO)</v>
       </c>
       <c r="C71" s="1356" t="inlineStr">
@@ -22378,75 +22020,57 @@
         </is>
       </c>
       <c r="D71" s="1357">
-        <f>'Para Histograma'!L589</f>
         <v>0</v>
       </c>
       <c r="E71" s="1357">
-        <f>'Para Histograma'!M589</f>
         <v>0</v>
       </c>
       <c r="F71" s="1357">
-        <f>'Para Histograma'!N589</f>
         <v>0</v>
       </c>
       <c r="G71" s="1357">
-        <f>'Para Histograma'!O589</f>
         <v>0</v>
       </c>
       <c r="H71" s="1357">
-        <f>'Para Histograma'!P589</f>
         <v>0</v>
       </c>
       <c r="I71" s="1357">
-        <f>'Para Histograma'!Q589</f>
         <v>0</v>
       </c>
       <c r="J71" s="1357">
-        <f>'Para Histograma'!R589</f>
         <v>0</v>
       </c>
       <c r="K71" s="1357">
-        <f>'Para Histograma'!S589</f>
         <v>0</v>
       </c>
       <c r="L71" s="1357">
-        <f>'Para Histograma'!T589</f>
         <v>0</v>
       </c>
       <c r="M71" s="1357">
-        <f>'Para Histograma'!U589</f>
         <v>0</v>
       </c>
       <c r="N71" s="1357">
-        <f>'Para Histograma'!V589</f>
         <v>1</v>
       </c>
       <c r="O71" s="1357">
-        <f>'Para Histograma'!W589</f>
         <v>1</v>
       </c>
       <c r="P71" s="1357">
-        <f>'Para Histograma'!X589</f>
         <v>1</v>
       </c>
       <c r="Q71" s="1357">
-        <f>'Para Histograma'!Y589</f>
         <v>1</v>
       </c>
       <c r="R71" s="1357">
-        <f>'Para Histograma'!Z589</f>
         <v>0</v>
       </c>
       <c r="S71" s="1357">
-        <f>'Para Histograma'!AA589</f>
         <v>0</v>
       </c>
       <c r="T71" s="1357">
-        <f>'Para Histograma'!AB589</f>
         <v>0</v>
       </c>
       <c r="U71" s="1357">
-        <f>'Para Histograma'!AC589</f>
         <v>0</v>
       </c>
     </row>
@@ -22510,75 +22134,57 @@
         </is>
       </c>
       <c r="D74" s="1364">
-        <f>SUMIF($C47:$C72,"Plan",D47:D72)</f>
         <v>0</v>
       </c>
       <c r="E74" s="1364">
-        <f t="shared" ref="E74:U74" si="4">SUMIF($C47:$C72,"Plan",E47:E72)</f>
         <v>0</v>
       </c>
       <c r="F74" s="1364">
-        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="G74" s="1364">
-        <f t="shared" si="4"/>
         <v>4</v>
       </c>
       <c r="H74" s="1364">
-        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="I74" s="1364">
-        <f t="shared" si="4"/>
         <v>11</v>
       </c>
       <c r="J74" s="1364">
-        <f t="shared" si="4"/>
         <v>12</v>
       </c>
       <c r="K74" s="1364">
-        <f t="shared" si="4"/>
         <v>14</v>
       </c>
       <c r="L74" s="1364">
-        <f t="shared" si="4"/>
         <v>18</v>
       </c>
       <c r="M74" s="1364">
-        <f t="shared" si="4"/>
         <v>17</v>
       </c>
       <c r="N74" s="1364">
-        <f t="shared" si="4"/>
         <v>20</v>
       </c>
       <c r="O74" s="1364">
-        <f t="shared" si="4"/>
         <v>20</v>
       </c>
       <c r="P74" s="1364">
-        <f t="shared" si="4"/>
         <v>20</v>
       </c>
       <c r="Q74" s="1364">
-        <f t="shared" si="4"/>
         <v>19</v>
       </c>
       <c r="R74" s="1364">
-        <f t="shared" si="4"/>
         <v>12</v>
       </c>
       <c r="S74" s="1364">
-        <f t="shared" si="4"/>
         <v>9</v>
       </c>
       <c r="T74" s="1364">
-        <f t="shared" si="4"/>
         <v>4</v>
       </c>
       <c r="U74" s="1364">
-        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -22590,75 +22196,57 @@
         </is>
       </c>
       <c r="D75" s="1492">
-        <f>SUMIF($C47:$C72,"Act.",D47:D72)</f>
         <v>0</v>
       </c>
       <c r="E75" s="1492">
-        <f t="shared" ref="E75:U75" si="5">SUMIF($C47:$C72,"Act.",E47:E72)</f>
         <v>0</v>
       </c>
       <c r="F75" s="1492">
-        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="G75" s="1492">
-        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="H75" s="1492">
-        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="I75" s="1492">
-        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="J75" s="1492">
-        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="K75" s="1492">
-        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="L75" s="1492">
-        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="M75" s="1492">
-        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="N75" s="1492">
-        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="O75" s="1492">
-        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="P75" s="1492">
-        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="Q75" s="1492">
-        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="R75" s="1492">
-        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="S75" s="1492">
-        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="T75" s="1492">
-        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="U75" s="1492">
-        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -22740,75 +22328,57 @@
         </is>
       </c>
       <c r="D79" s="1373">
-        <f t="shared" ref="D79:O79" si="6">D26+D42+D74</f>
         <v>16</v>
       </c>
       <c r="E79" s="1373">
-        <f t="shared" si="6"/>
         <v>16</v>
       </c>
       <c r="F79" s="1373">
-        <f t="shared" si="6"/>
         <v>17</v>
       </c>
       <c r="G79" s="1373">
-        <f t="shared" si="6"/>
         <v>20</v>
       </c>
       <c r="H79" s="1373">
-        <f t="shared" si="6"/>
         <v>21</v>
       </c>
       <c r="I79" s="1373">
-        <f t="shared" si="6"/>
         <v>27</v>
       </c>
       <c r="J79" s="1373">
-        <f t="shared" si="6"/>
         <v>28</v>
       </c>
       <c r="K79" s="1373">
-        <f t="shared" si="6"/>
         <v>30</v>
       </c>
       <c r="L79" s="1373">
-        <f t="shared" si="6"/>
         <v>34</v>
       </c>
       <c r="M79" s="1373">
-        <f t="shared" si="6"/>
         <v>33</v>
       </c>
       <c r="N79" s="1373">
-        <f t="shared" si="6"/>
         <v>36</v>
       </c>
       <c r="O79" s="1373">
-        <f t="shared" si="6"/>
         <v>36</v>
       </c>
       <c r="P79" s="1373">
-        <f t="shared" ref="P79:U79" si="7">P26+P42+P74</f>
         <v>36</v>
       </c>
       <c r="Q79" s="1373">
-        <f t="shared" si="7"/>
         <v>35</v>
       </c>
       <c r="R79" s="1373">
-        <f t="shared" si="7"/>
         <v>28</v>
       </c>
       <c r="S79" s="1373">
-        <f t="shared" si="7"/>
         <v>25</v>
       </c>
       <c r="T79" s="1373">
-        <f t="shared" si="7"/>
         <v>20</v>
       </c>
       <c r="U79" s="1373">
-        <f t="shared" si="7"/>
         <v>16</v>
       </c>
     </row>
@@ -22820,75 +22390,57 @@
         </is>
       </c>
       <c r="D80" s="1492">
-        <f t="shared" ref="D80:O80" si="8">D27+D43+D75</f>
         <v>0</v>
       </c>
       <c r="E80" s="1492">
-        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F80" s="1492">
-        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="G80" s="1492">
-        <f t="shared" si="8"/>
         <v>14</v>
       </c>
       <c r="H80" s="1492">
-        <f t="shared" si="8"/>
         <v>15</v>
       </c>
       <c r="I80" s="1492">
-        <f t="shared" si="8"/>
         <v>15</v>
       </c>
       <c r="J80" s="1492">
-        <f t="shared" si="8"/>
         <v>15</v>
       </c>
       <c r="K80" s="1492">
-        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="L80" s="1492">
-        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M80" s="1492">
-        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="N80" s="1492">
-        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="O80" s="1492">
-        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="P80" s="1492">
-        <f t="shared" ref="P80:U80" si="9">P27+P43+P75</f>
         <v>0</v>
       </c>
       <c r="Q80" s="1492">
-        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="R80" s="1492">
-        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="S80" s="1492">
-        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="T80" s="1492">
-        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="U80" s="1492">
-        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -22991,7 +22543,6 @@
         </is>
       </c>
       <c r="C4" s="1345">
-        <f>'STAFFING TABULATION CHART'!C4</f>
         <v>0</v>
       </c>
     </row>
@@ -23002,7 +22553,6 @@
         </is>
       </c>
       <c r="C5" s="1345" t="str">
-        <f>'STAFFING TABULATION CHART'!C5</f>
         <v>CONSORCIO CPQ COLUMBITO</v>
       </c>
     </row>
@@ -23013,7 +22563,6 @@
         </is>
       </c>
       <c r="C6" s="1345" t="str">
-        <f>'STAFFING TABULATION CHART'!C6</f>
         <v>REPOSICION DEL SISTEMA DE FLOCULANTES — LB0</v>
       </c>
     </row>
@@ -23028,224 +22577,170 @@
     <row r="9" spans="2:21" s="1348" customFormat="1">
       <c r="B9" s="1344"/>
       <c r="D9" s="1374">
-        <f>'PHYSICAL % PROGRESS'!P7</f>
         <v>27</v>
       </c>
       <c r="E9" s="1374">
-        <f>'PHYSICAL % PROGRESS'!Q7</f>
         <v>28</v>
       </c>
       <c r="F9" s="1374">
-        <f>'PHYSICAL % PROGRESS'!R7</f>
         <v>29</v>
       </c>
       <c r="G9" s="1374">
-        <f>'PHYSICAL % PROGRESS'!S7</f>
         <v>30</v>
       </c>
       <c r="H9" s="1374">
-        <f>'PHYSICAL % PROGRESS'!T7</f>
         <v>31</v>
       </c>
       <c r="I9" s="1374">
-        <f>'PHYSICAL % PROGRESS'!U7</f>
         <v>32</v>
       </c>
       <c r="J9" s="1374">
-        <f>'PHYSICAL % PROGRESS'!V7</f>
         <v>33</v>
       </c>
       <c r="K9" s="1374">
-        <f>'PHYSICAL % PROGRESS'!W7</f>
         <v>34</v>
       </c>
       <c r="L9" s="1374">
-        <f>'PHYSICAL % PROGRESS'!X7</f>
         <v>35</v>
       </c>
       <c r="M9" s="1374">
-        <f>'PHYSICAL % PROGRESS'!Y7</f>
         <v>36</v>
       </c>
       <c r="N9" s="1374">
-        <f>'PHYSICAL % PROGRESS'!Z7</f>
         <v>37</v>
       </c>
       <c r="O9" s="1374">
-        <f>'PHYSICAL % PROGRESS'!AA7</f>
         <v>38</v>
       </c>
       <c r="P9" s="1374">
-        <f>'PHYSICAL % PROGRESS'!AB7</f>
         <v>39</v>
       </c>
       <c r="Q9" s="1374">
-        <f>'PHYSICAL % PROGRESS'!AC7</f>
         <v>40</v>
       </c>
       <c r="R9" s="1374">
-        <f>'PHYSICAL % PROGRESS'!AD7</f>
         <v>41</v>
       </c>
       <c r="S9" s="1374">
-        <f>'PHYSICAL % PROGRESS'!AE7</f>
         <v>42</v>
       </c>
       <c r="T9" s="1374">
-        <f>'PHYSICAL % PROGRESS'!AF7</f>
         <v>43</v>
       </c>
       <c r="U9" s="1374">
-        <f>'PHYSICAL % PROGRESS'!AG7</f>
         <v>44</v>
       </c>
     </row>
     <row r="10" spans="2:21" s="1348" customFormat="1">
       <c r="B10" s="1344"/>
       <c r="D10" s="1375">
-        <f>'PHYSICAL % PROGRESS'!P8</f>
         <v>46199</v>
       </c>
       <c r="E10" s="1375">
-        <f>'PHYSICAL % PROGRESS'!Q8</f>
         <v>46206</v>
       </c>
       <c r="F10" s="1375">
-        <f>'PHYSICAL % PROGRESS'!R8</f>
         <v>46213</v>
       </c>
       <c r="G10" s="1375">
-        <f>'PHYSICAL % PROGRESS'!S8</f>
         <v>46220</v>
       </c>
       <c r="H10" s="1375">
-        <f>'PHYSICAL % PROGRESS'!T8</f>
         <v>46227</v>
       </c>
       <c r="I10" s="1375">
-        <f>'PHYSICAL % PROGRESS'!U8</f>
         <v>46234</v>
       </c>
       <c r="J10" s="1375">
-        <f>'PHYSICAL % PROGRESS'!V8</f>
         <v>46241</v>
       </c>
       <c r="K10" s="1375">
-        <f>'PHYSICAL % PROGRESS'!W8</f>
         <v>46248</v>
       </c>
       <c r="L10" s="1375">
-        <f>'PHYSICAL % PROGRESS'!X8</f>
         <v>46255</v>
       </c>
       <c r="M10" s="1375">
-        <f>'PHYSICAL % PROGRESS'!Y8</f>
         <v>46262</v>
       </c>
       <c r="N10" s="1375">
-        <f>'PHYSICAL % PROGRESS'!Z8</f>
         <v>46269</v>
       </c>
       <c r="O10" s="1375">
-        <f>'PHYSICAL % PROGRESS'!AA8</f>
         <v>46276</v>
       </c>
       <c r="P10" s="1375">
-        <f>'PHYSICAL % PROGRESS'!AB8</f>
         <v>46283</v>
       </c>
       <c r="Q10" s="1375">
-        <f>'PHYSICAL % PROGRESS'!AC8</f>
         <v>46290</v>
       </c>
       <c r="R10" s="1375">
-        <f>'PHYSICAL % PROGRESS'!AD8</f>
         <v>46297</v>
       </c>
       <c r="S10" s="1375">
-        <f>'PHYSICAL % PROGRESS'!AE8</f>
         <v>46304</v>
       </c>
       <c r="T10" s="1375">
-        <f>'PHYSICAL % PROGRESS'!AF8</f>
         <v>46311</v>
       </c>
       <c r="U10" s="1375">
-        <f>'PHYSICAL % PROGRESS'!AG8</f>
         <v>46318</v>
       </c>
     </row>
     <row r="11" spans="2:21" s="1348" customFormat="1">
       <c r="D11" s="1376">
-        <f>'PHYSICAL % PROGRESS'!P9</f>
         <v>46205</v>
       </c>
       <c r="E11" s="1376">
-        <f>'PHYSICAL % PROGRESS'!Q9</f>
         <v>46212</v>
       </c>
       <c r="F11" s="1376">
-        <f>'PHYSICAL % PROGRESS'!R9</f>
         <v>46219</v>
       </c>
       <c r="G11" s="1376">
-        <f>'PHYSICAL % PROGRESS'!S9</f>
         <v>46226</v>
       </c>
       <c r="H11" s="1376">
-        <f>'PHYSICAL % PROGRESS'!T9</f>
         <v>46233</v>
       </c>
       <c r="I11" s="1376">
-        <f>'PHYSICAL % PROGRESS'!U9</f>
         <v>46240</v>
       </c>
       <c r="J11" s="1376">
-        <f>'PHYSICAL % PROGRESS'!V9</f>
         <v>46247</v>
       </c>
       <c r="K11" s="1376">
-        <f>'PHYSICAL % PROGRESS'!W9</f>
         <v>46254</v>
       </c>
       <c r="L11" s="1376">
-        <f>'PHYSICAL % PROGRESS'!X9</f>
         <v>46261</v>
       </c>
       <c r="M11" s="1376">
-        <f>'PHYSICAL % PROGRESS'!Y9</f>
         <v>46268</v>
       </c>
       <c r="N11" s="1376">
-        <f>'PHYSICAL % PROGRESS'!Z9</f>
         <v>46275</v>
       </c>
       <c r="O11" s="1376">
-        <f>'PHYSICAL % PROGRESS'!AA9</f>
         <v>46282</v>
       </c>
       <c r="P11" s="1376">
-        <f>'PHYSICAL % PROGRESS'!AB9</f>
         <v>46289</v>
       </c>
       <c r="Q11" s="1376">
-        <f>'PHYSICAL % PROGRESS'!AC9</f>
         <v>46296</v>
       </c>
       <c r="R11" s="1376">
-        <f>'PHYSICAL % PROGRESS'!AD9</f>
         <v>46303</v>
       </c>
       <c r="S11" s="1376">
-        <f>'PHYSICAL % PROGRESS'!AE9</f>
         <v>46310</v>
       </c>
       <c r="T11" s="1376">
-        <f>'PHYSICAL % PROGRESS'!AF9</f>
         <v>46317</v>
       </c>
       <c r="U11" s="1376">
-        <f>'PHYSICAL % PROGRESS'!AG9</f>
         <v>46324</v>
       </c>
     </row>
@@ -23277,7 +22772,6 @@
     </row>
     <row r="13" spans="2:21" s="1379" customFormat="1">
       <c r="B13" s="1500" t="str">
-        <f>'Para Histograma'!D599</f>
         <v>CAMION GRUA DE 12TN</v>
       </c>
       <c r="C13" s="1356" t="inlineStr">
@@ -23286,75 +22780,57 @@
         </is>
       </c>
       <c r="D13" s="1357">
-        <f>'Para Histograma'!L599</f>
         <v>0</v>
       </c>
       <c r="E13" s="1357">
-        <f>'Para Histograma'!M599</f>
         <v>0</v>
       </c>
       <c r="F13" s="1357">
-        <f>'Para Histograma'!N599</f>
         <v>0</v>
       </c>
       <c r="G13" s="1357">
-        <f>'Para Histograma'!O599</f>
         <v>1</v>
       </c>
       <c r="H13" s="1357">
-        <f>'Para Histograma'!P599</f>
         <v>0</v>
       </c>
       <c r="I13" s="1357">
-        <f>'Para Histograma'!Q599</f>
         <v>0</v>
       </c>
       <c r="J13" s="1357">
-        <f>'Para Histograma'!R599</f>
         <v>0</v>
       </c>
       <c r="K13" s="1357">
-        <f>'Para Histograma'!S599</f>
         <v>0</v>
       </c>
       <c r="L13" s="1357">
-        <f>'Para Histograma'!T599</f>
         <v>0</v>
       </c>
       <c r="M13" s="1357">
-        <f>'Para Histograma'!U599</f>
         <v>0</v>
       </c>
       <c r="N13" s="1357">
-        <f>'Para Histograma'!V599</f>
         <v>0</v>
       </c>
       <c r="O13" s="1357">
-        <f>'Para Histograma'!W599</f>
         <v>0</v>
       </c>
       <c r="P13" s="1357">
-        <f>'Para Histograma'!X599</f>
         <v>0</v>
       </c>
       <c r="Q13" s="1357">
-        <f>'Para Histograma'!Y599</f>
         <v>0</v>
       </c>
       <c r="R13" s="1357">
-        <f>'Para Histograma'!Z599</f>
         <v>0</v>
       </c>
       <c r="S13" s="1357">
-        <f>'Para Histograma'!AA599</f>
         <v>0</v>
       </c>
       <c r="T13" s="1357">
-        <f>'Para Histograma'!AB599</f>
         <v>0</v>
       </c>
       <c r="U13" s="1357">
-        <f>'Para Histograma'!AC599</f>
         <v>0</v>
       </c>
     </row>
@@ -23386,7 +22862,6 @@
     </row>
     <row r="15" spans="2:21" s="1379" customFormat="1">
       <c r="B15" s="1500" t="str">
-        <f>'Para Histograma'!D600</f>
         <v>CAMION BARANDA (4TN)</v>
       </c>
       <c r="C15" s="1356" t="inlineStr">
@@ -23395,75 +22870,57 @@
         </is>
       </c>
       <c r="D15" s="1357">
-        <f>'Para Histograma'!L600</f>
         <v>0</v>
       </c>
       <c r="E15" s="1357">
-        <f>'Para Histograma'!M600</f>
         <v>0</v>
       </c>
       <c r="F15" s="1357">
-        <f>'Para Histograma'!N600</f>
         <v>0</v>
       </c>
       <c r="G15" s="1357">
-        <f>'Para Histograma'!O600</f>
         <v>1</v>
       </c>
       <c r="H15" s="1357">
-        <f>'Para Histograma'!P600</f>
         <v>0</v>
       </c>
       <c r="I15" s="1357">
-        <f>'Para Histograma'!Q600</f>
         <v>0</v>
       </c>
       <c r="J15" s="1357">
-        <f>'Para Histograma'!R600</f>
         <v>0</v>
       </c>
       <c r="K15" s="1357">
-        <f>'Para Histograma'!S600</f>
         <v>0</v>
       </c>
       <c r="L15" s="1357">
-        <f>'Para Histograma'!T600</f>
         <v>0</v>
       </c>
       <c r="M15" s="1357">
-        <f>'Para Histograma'!U600</f>
         <v>0</v>
       </c>
       <c r="N15" s="1357">
-        <f>'Para Histograma'!V600</f>
         <v>0</v>
       </c>
       <c r="O15" s="1357">
-        <f>'Para Histograma'!W600</f>
         <v>0</v>
       </c>
       <c r="P15" s="1357">
-        <f>'Para Histograma'!X600</f>
         <v>0</v>
       </c>
       <c r="Q15" s="1357">
-        <f>'Para Histograma'!Y600</f>
         <v>0</v>
       </c>
       <c r="R15" s="1357">
-        <f>'Para Histograma'!Z600</f>
         <v>0</v>
       </c>
       <c r="S15" s="1357">
-        <f>'Para Histograma'!AA600</f>
         <v>0</v>
       </c>
       <c r="T15" s="1357">
-        <f>'Para Histograma'!AB600</f>
         <v>0</v>
       </c>
       <c r="U15" s="1357">
-        <f>'Para Histograma'!AC600</f>
         <v>0</v>
       </c>
     </row>
@@ -23495,7 +22952,6 @@
     </row>
     <row r="17" spans="2:21" s="1379" customFormat="1">
       <c r="B17" s="1500" t="str">
-        <f>'Para Histograma'!D601</f>
         <v>NIVEL DE INGENIERO</v>
       </c>
       <c r="C17" s="1356" t="inlineStr">
@@ -23504,75 +22960,57 @@
         </is>
       </c>
       <c r="D17" s="1357">
-        <f>'Para Histograma'!L601</f>
         <v>0</v>
       </c>
       <c r="E17" s="1357">
-        <f>'Para Histograma'!M601</f>
         <v>0</v>
       </c>
       <c r="F17" s="1357">
-        <f>'Para Histograma'!N601</f>
         <v>0</v>
       </c>
       <c r="G17" s="1357">
-        <f>'Para Histograma'!O601</f>
         <v>0</v>
       </c>
       <c r="H17" s="1357">
-        <f>'Para Histograma'!P601</f>
         <v>1</v>
       </c>
       <c r="I17" s="1357">
-        <f>'Para Histograma'!Q601</f>
         <v>0</v>
       </c>
       <c r="J17" s="1357">
-        <f>'Para Histograma'!R601</f>
         <v>0</v>
       </c>
       <c r="K17" s="1357">
-        <f>'Para Histograma'!S601</f>
         <v>0</v>
       </c>
       <c r="L17" s="1357">
-        <f>'Para Histograma'!T601</f>
         <v>0</v>
       </c>
       <c r="M17" s="1357">
-        <f>'Para Histograma'!U601</f>
         <v>0</v>
       </c>
       <c r="N17" s="1357">
-        <f>'Para Histograma'!V601</f>
         <v>0</v>
       </c>
       <c r="O17" s="1357">
-        <f>'Para Histograma'!W601</f>
         <v>0</v>
       </c>
       <c r="P17" s="1357">
-        <f>'Para Histograma'!X601</f>
         <v>0</v>
       </c>
       <c r="Q17" s="1357">
-        <f>'Para Histograma'!Y601</f>
         <v>0</v>
       </c>
       <c r="R17" s="1357">
-        <f>'Para Histograma'!Z601</f>
         <v>0</v>
       </c>
       <c r="S17" s="1357">
-        <f>'Para Histograma'!AA601</f>
         <v>0</v>
       </c>
       <c r="T17" s="1357">
-        <f>'Para Histograma'!AB601</f>
         <v>0</v>
       </c>
       <c r="U17" s="1357">
-        <f>'Para Histograma'!AC601</f>
         <v>0</v>
       </c>
     </row>
@@ -23604,7 +23042,6 @@
     </row>
     <row r="19" spans="2:21" s="1379" customFormat="1">
       <c r="B19" s="1500" t="str">
-        <f>'Para Histograma'!D602</f>
         <v xml:space="preserve">ROTOMARTILLO </v>
       </c>
       <c r="C19" s="1356" t="inlineStr">
@@ -23613,75 +23050,57 @@
         </is>
       </c>
       <c r="D19" s="1357">
-        <f>'Para Histograma'!L602</f>
         <v>0</v>
       </c>
       <c r="E19" s="1357">
-        <f>'Para Histograma'!M602</f>
         <v>0</v>
       </c>
       <c r="F19" s="1357">
-        <f>'Para Histograma'!N602</f>
         <v>0</v>
       </c>
       <c r="G19" s="1357">
-        <f>'Para Histograma'!O602</f>
         <v>0</v>
       </c>
       <c r="H19" s="1357">
-        <f>'Para Histograma'!P602</f>
         <v>1</v>
       </c>
       <c r="I19" s="1357">
-        <f>'Para Histograma'!Q602</f>
         <v>0</v>
       </c>
       <c r="J19" s="1357">
-        <f>'Para Histograma'!R602</f>
         <v>0</v>
       </c>
       <c r="K19" s="1357">
-        <f>'Para Histograma'!S602</f>
         <v>0</v>
       </c>
       <c r="L19" s="1357">
-        <f>'Para Histograma'!T602</f>
         <v>0</v>
       </c>
       <c r="M19" s="1357">
-        <f>'Para Histograma'!U602</f>
         <v>0</v>
       </c>
       <c r="N19" s="1357">
-        <f>'Para Histograma'!V602</f>
         <v>0</v>
       </c>
       <c r="O19" s="1357">
-        <f>'Para Histograma'!W602</f>
         <v>0</v>
       </c>
       <c r="P19" s="1357">
-        <f>'Para Histograma'!X602</f>
         <v>0</v>
       </c>
       <c r="Q19" s="1357">
-        <f>'Para Histograma'!Y602</f>
         <v>0</v>
       </c>
       <c r="R19" s="1357">
-        <f>'Para Histograma'!Z602</f>
         <v>0</v>
       </c>
       <c r="S19" s="1357">
-        <f>'Para Histograma'!AA602</f>
         <v>0</v>
       </c>
       <c r="T19" s="1357">
-        <f>'Para Histograma'!AB602</f>
         <v>0</v>
       </c>
       <c r="U19" s="1357">
-        <f>'Para Histograma'!AC602</f>
         <v>0</v>
       </c>
     </row>
@@ -23713,7 +23132,6 @@
     </row>
     <row r="21" spans="2:21" s="1379" customFormat="1">
       <c r="B21" s="1500" t="str">
-        <f>'Para Histograma'!D603</f>
         <v xml:space="preserve">VIBRADORA DE CONCRETO </v>
       </c>
       <c r="C21" s="1356" t="inlineStr">
@@ -23722,75 +23140,57 @@
         </is>
       </c>
       <c r="D21" s="1357">
-        <f>'Para Histograma'!L603</f>
         <v>0</v>
       </c>
       <c r="E21" s="1357">
-        <f>'Para Histograma'!M603</f>
         <v>0</v>
       </c>
       <c r="F21" s="1357">
-        <f>'Para Histograma'!N603</f>
         <v>0</v>
       </c>
       <c r="G21" s="1357">
-        <f>'Para Histograma'!O603</f>
         <v>0</v>
       </c>
       <c r="H21" s="1357">
-        <f>'Para Histograma'!P603</f>
         <v>0</v>
       </c>
       <c r="I21" s="1357">
-        <f>'Para Histograma'!Q603</f>
         <v>1</v>
       </c>
       <c r="J21" s="1357">
-        <f>'Para Histograma'!R603</f>
         <v>0</v>
       </c>
       <c r="K21" s="1357">
-        <f>'Para Histograma'!S603</f>
         <v>0</v>
       </c>
       <c r="L21" s="1357">
-        <f>'Para Histograma'!T603</f>
         <v>0</v>
       </c>
       <c r="M21" s="1357">
-        <f>'Para Histograma'!U603</f>
         <v>0</v>
       </c>
       <c r="N21" s="1357">
-        <f>'Para Histograma'!V603</f>
         <v>0</v>
       </c>
       <c r="O21" s="1357">
-        <f>'Para Histograma'!W603</f>
         <v>0</v>
       </c>
       <c r="P21" s="1357">
-        <f>'Para Histograma'!X603</f>
         <v>0</v>
       </c>
       <c r="Q21" s="1357">
-        <f>'Para Histograma'!Y603</f>
         <v>0</v>
       </c>
       <c r="R21" s="1357">
-        <f>'Para Histograma'!Z603</f>
         <v>0</v>
       </c>
       <c r="S21" s="1357">
-        <f>'Para Histograma'!AA603</f>
         <v>0</v>
       </c>
       <c r="T21" s="1357">
-        <f>'Para Histograma'!AB603</f>
         <v>0</v>
       </c>
       <c r="U21" s="1357">
-        <f>'Para Histograma'!AC603</f>
         <v>0</v>
       </c>
     </row>
@@ -23822,7 +23222,6 @@
     </row>
     <row r="23" spans="2:21" s="1379" customFormat="1">
       <c r="B23" s="1500" t="str">
-        <f>'Para Histograma'!D604</f>
         <v>SIERRA CIRCULAR</v>
       </c>
       <c r="C23" s="1356" t="inlineStr">
@@ -23831,75 +23230,57 @@
         </is>
       </c>
       <c r="D23" s="1357">
-        <f>'Para Histograma'!L604</f>
         <v>0</v>
       </c>
       <c r="E23" s="1357">
-        <f>'Para Histograma'!M604</f>
         <v>0</v>
       </c>
       <c r="F23" s="1357">
-        <f>'Para Histograma'!N604</f>
         <v>0</v>
       </c>
       <c r="G23" s="1357">
-        <f>'Para Histograma'!O604</f>
         <v>0</v>
       </c>
       <c r="H23" s="1357">
-        <f>'Para Histograma'!P604</f>
         <v>0</v>
       </c>
       <c r="I23" s="1357">
-        <f>'Para Histograma'!Q604</f>
         <v>0</v>
       </c>
       <c r="J23" s="1357">
-        <f>'Para Histograma'!R604</f>
         <v>1</v>
       </c>
       <c r="K23" s="1357">
-        <f>'Para Histograma'!S604</f>
         <v>0</v>
       </c>
       <c r="L23" s="1357">
-        <f>'Para Histograma'!T604</f>
         <v>0</v>
       </c>
       <c r="M23" s="1357">
-        <f>'Para Histograma'!U604</f>
         <v>0</v>
       </c>
       <c r="N23" s="1357">
-        <f>'Para Histograma'!V604</f>
         <v>0</v>
       </c>
       <c r="O23" s="1357">
-        <f>'Para Histograma'!W604</f>
         <v>0</v>
       </c>
       <c r="P23" s="1357">
-        <f>'Para Histograma'!X604</f>
         <v>0</v>
       </c>
       <c r="Q23" s="1357">
-        <f>'Para Histograma'!Y604</f>
         <v>0</v>
       </c>
       <c r="R23" s="1357">
-        <f>'Para Histograma'!Z604</f>
         <v>0</v>
       </c>
       <c r="S23" s="1357">
-        <f>'Para Histograma'!AA604</f>
         <v>0</v>
       </c>
       <c r="T23" s="1357">
-        <f>'Para Histograma'!AB604</f>
         <v>0</v>
       </c>
       <c r="U23" s="1357">
-        <f>'Para Histograma'!AC604</f>
         <v>0</v>
       </c>
     </row>
@@ -23931,7 +23312,6 @@
     </row>
     <row r="25" spans="2:21" s="1379" customFormat="1">
       <c r="B25" s="1500" t="str">
-        <f>'Para Histograma'!D605</f>
         <v xml:space="preserve">ESMERIL ELÉCTRICO </v>
       </c>
       <c r="C25" s="1356" t="inlineStr">
@@ -23940,75 +23320,57 @@
         </is>
       </c>
       <c r="D25" s="1357">
-        <f>'Para Histograma'!L605</f>
         <v>0</v>
       </c>
       <c r="E25" s="1357">
-        <f>'Para Histograma'!M605</f>
         <v>0</v>
       </c>
       <c r="F25" s="1357">
-        <f>'Para Histograma'!N605</f>
         <v>0</v>
       </c>
       <c r="G25" s="1357">
-        <f>'Para Histograma'!O605</f>
         <v>0</v>
       </c>
       <c r="H25" s="1357">
-        <f>'Para Histograma'!P605</f>
         <v>0</v>
       </c>
       <c r="I25" s="1357">
-        <f>'Para Histograma'!Q605</f>
         <v>0</v>
       </c>
       <c r="J25" s="1357">
-        <f>'Para Histograma'!R605</f>
         <v>1</v>
       </c>
       <c r="K25" s="1357">
-        <f>'Para Histograma'!S605</f>
         <v>0</v>
       </c>
       <c r="L25" s="1357">
-        <f>'Para Histograma'!T605</f>
         <v>0</v>
       </c>
       <c r="M25" s="1357">
-        <f>'Para Histograma'!U605</f>
         <v>0</v>
       </c>
       <c r="N25" s="1357">
-        <f>'Para Histograma'!V605</f>
         <v>0</v>
       </c>
       <c r="O25" s="1357">
-        <f>'Para Histograma'!W605</f>
         <v>0</v>
       </c>
       <c r="P25" s="1357">
-        <f>'Para Histograma'!X605</f>
         <v>0</v>
       </c>
       <c r="Q25" s="1357">
-        <f>'Para Histograma'!Y605</f>
         <v>0</v>
       </c>
       <c r="R25" s="1357">
-        <f>'Para Histograma'!Z605</f>
         <v>0</v>
       </c>
       <c r="S25" s="1357">
-        <f>'Para Histograma'!AA605</f>
         <v>0</v>
       </c>
       <c r="T25" s="1357">
-        <f>'Para Histograma'!AB605</f>
         <v>0</v>
       </c>
       <c r="U25" s="1357">
-        <f>'Para Histograma'!AC605</f>
         <v>0</v>
       </c>
     </row>
@@ -24040,7 +23402,6 @@
     </row>
     <row r="27" spans="2:21" s="1379" customFormat="1">
       <c r="B27" s="1500" t="str">
-        <f>'Para Histograma'!D606</f>
         <v>AMOLADORA</v>
       </c>
       <c r="C27" s="1356" t="inlineStr">
@@ -24049,75 +23410,57 @@
         </is>
       </c>
       <c r="D27" s="1357">
-        <f>'Para Histograma'!L606</f>
         <v>0</v>
       </c>
       <c r="E27" s="1357">
-        <f>'Para Histograma'!M606</f>
         <v>0</v>
       </c>
       <c r="F27" s="1357">
-        <f>'Para Histograma'!N606</f>
         <v>0</v>
       </c>
       <c r="G27" s="1357">
-        <f>'Para Histograma'!O606</f>
         <v>0</v>
       </c>
       <c r="H27" s="1357">
-        <f>'Para Histograma'!P606</f>
         <v>0</v>
       </c>
       <c r="I27" s="1357">
-        <f>'Para Histograma'!Q606</f>
         <v>1</v>
       </c>
       <c r="J27" s="1357">
-        <f>'Para Histograma'!R606</f>
         <v>1</v>
       </c>
       <c r="K27" s="1357">
-        <f>'Para Histograma'!S606</f>
         <v>1</v>
       </c>
       <c r="L27" s="1357">
-        <f>'Para Histograma'!T606</f>
         <v>1</v>
       </c>
       <c r="M27" s="1357">
-        <f>'Para Histograma'!U606</f>
         <v>0</v>
       </c>
       <c r="N27" s="1357">
-        <f>'Para Histograma'!V606</f>
         <v>0</v>
       </c>
       <c r="O27" s="1357">
-        <f>'Para Histograma'!W606</f>
         <v>0</v>
       </c>
       <c r="P27" s="1357">
-        <f>'Para Histograma'!X606</f>
         <v>0</v>
       </c>
       <c r="Q27" s="1357">
-        <f>'Para Histograma'!Y606</f>
         <v>0</v>
       </c>
       <c r="R27" s="1357">
-        <f>'Para Histograma'!Z606</f>
         <v>0</v>
       </c>
       <c r="S27" s="1357">
-        <f>'Para Histograma'!AA606</f>
         <v>0</v>
       </c>
       <c r="T27" s="1357">
-        <f>'Para Histograma'!AB606</f>
         <v>0</v>
       </c>
       <c r="U27" s="1357">
-        <f>'Para Histograma'!AC606</f>
         <v>0</v>
       </c>
     </row>
@@ -24149,7 +23492,6 @@
     </row>
     <row r="29" spans="2:21" s="1379" customFormat="1">
       <c r="B29" s="1500" t="str">
-        <f>'Para Histograma'!D607</f>
         <v xml:space="preserve">COMPRESORA </v>
       </c>
       <c r="C29" s="1356" t="inlineStr">
@@ -24158,75 +23500,57 @@
         </is>
       </c>
       <c r="D29" s="1357">
-        <f>'Para Histograma'!L607</f>
         <v>0</v>
       </c>
       <c r="E29" s="1357">
-        <f>'Para Histograma'!M607</f>
         <v>0</v>
       </c>
       <c r="F29" s="1357">
-        <f>'Para Histograma'!N607</f>
         <v>0</v>
       </c>
       <c r="G29" s="1357">
-        <f>'Para Histograma'!O607</f>
         <v>0</v>
       </c>
       <c r="H29" s="1357">
-        <f>'Para Histograma'!P607</f>
         <v>0</v>
       </c>
       <c r="I29" s="1357">
-        <f>'Para Histograma'!Q607</f>
         <v>0</v>
       </c>
       <c r="J29" s="1357">
-        <f>'Para Histograma'!R607</f>
         <v>0</v>
       </c>
       <c r="K29" s="1357">
-        <f>'Para Histograma'!S607</f>
         <v>0</v>
       </c>
       <c r="L29" s="1357">
-        <f>'Para Histograma'!T607</f>
         <v>0</v>
       </c>
       <c r="M29" s="1357">
-        <f>'Para Histograma'!U607</f>
         <v>1</v>
       </c>
       <c r="N29" s="1357">
-        <f>'Para Histograma'!V607</f>
         <v>0</v>
       </c>
       <c r="O29" s="1357">
-        <f>'Para Histograma'!W607</f>
         <v>0</v>
       </c>
       <c r="P29" s="1357">
-        <f>'Para Histograma'!X607</f>
         <v>0</v>
       </c>
       <c r="Q29" s="1357">
-        <f>'Para Histograma'!Y607</f>
         <v>0</v>
       </c>
       <c r="R29" s="1357">
-        <f>'Para Histograma'!Z607</f>
         <v>0</v>
       </c>
       <c r="S29" s="1357">
-        <f>'Para Histograma'!AA607</f>
         <v>0</v>
       </c>
       <c r="T29" s="1357">
-        <f>'Para Histograma'!AB607</f>
         <v>0</v>
       </c>
       <c r="U29" s="1357">
-        <f>'Para Histograma'!AC607</f>
         <v>0</v>
       </c>
     </row>
@@ -24258,7 +23582,6 @@
     </row>
     <row r="31" spans="2:21" s="1379" customFormat="1">
       <c r="B31" s="1500" t="str">
-        <f>'Para Histograma'!D608</f>
         <v>MAQUINA DE SOLDAR</v>
       </c>
       <c r="C31" s="1356" t="inlineStr">
@@ -24267,75 +23590,57 @@
         </is>
       </c>
       <c r="D31" s="1357">
-        <f>'Para Histograma'!L608</f>
         <v>0</v>
       </c>
       <c r="E31" s="1357">
-        <f>'Para Histograma'!M608</f>
         <v>0</v>
       </c>
       <c r="F31" s="1357">
-        <f>'Para Histograma'!N608</f>
         <v>0</v>
       </c>
       <c r="G31" s="1357">
-        <f>'Para Histograma'!O608</f>
         <v>0</v>
       </c>
       <c r="H31" s="1357">
-        <f>'Para Histograma'!P608</f>
         <v>0</v>
       </c>
       <c r="I31" s="1357">
-        <f>'Para Histograma'!Q608</f>
         <v>0</v>
       </c>
       <c r="J31" s="1357">
-        <f>'Para Histograma'!R608</f>
         <v>0</v>
       </c>
       <c r="K31" s="1357">
-        <f>'Para Histograma'!S608</f>
         <v>2</v>
       </c>
       <c r="L31" s="1357">
-        <f>'Para Histograma'!T608</f>
         <v>2</v>
       </c>
       <c r="M31" s="1357">
-        <f>'Para Histograma'!U608</f>
         <v>2</v>
       </c>
       <c r="N31" s="1357">
-        <f>'Para Histograma'!V608</f>
         <v>2</v>
       </c>
       <c r="O31" s="1357">
-        <f>'Para Histograma'!W608</f>
         <v>3</v>
       </c>
       <c r="P31" s="1357">
-        <f>'Para Histograma'!X608</f>
         <v>2</v>
       </c>
       <c r="Q31" s="1357">
-        <f>'Para Histograma'!Y608</f>
         <v>2</v>
       </c>
       <c r="R31" s="1357">
-        <f>'Para Histograma'!Z608</f>
         <v>2</v>
       </c>
       <c r="S31" s="1357">
-        <f>'Para Histograma'!AA608</f>
         <v>1</v>
       </c>
       <c r="T31" s="1357">
-        <f>'Para Histograma'!AB608</f>
         <v>1</v>
       </c>
       <c r="U31" s="1357">
-        <f>'Para Histograma'!AC608</f>
         <v>0</v>
       </c>
     </row>
@@ -24367,7 +23672,6 @@
     </row>
     <row r="33" spans="2:21" s="1379" customFormat="1">
       <c r="B33" s="1500" t="str">
-        <f>'Para Histograma'!D609</f>
         <v>BATIDORA DE GROUT</v>
       </c>
       <c r="C33" s="1356" t="inlineStr">
@@ -24376,75 +23680,57 @@
         </is>
       </c>
       <c r="D33" s="1357">
-        <f>'Para Histograma'!L609</f>
         <v>0</v>
       </c>
       <c r="E33" s="1357">
-        <f>'Para Histograma'!M609</f>
         <v>0</v>
       </c>
       <c r="F33" s="1357">
-        <f>'Para Histograma'!N609</f>
         <v>0</v>
       </c>
       <c r="G33" s="1357">
-        <f>'Para Histograma'!O609</f>
         <v>0</v>
       </c>
       <c r="H33" s="1357">
-        <f>'Para Histograma'!P609</f>
         <v>0</v>
       </c>
       <c r="I33" s="1357">
-        <f>'Para Histograma'!Q609</f>
         <v>0</v>
       </c>
       <c r="J33" s="1357">
-        <f>'Para Histograma'!R609</f>
         <v>0</v>
       </c>
       <c r="K33" s="1357">
-        <f>'Para Histograma'!S609</f>
         <v>0</v>
       </c>
       <c r="L33" s="1357">
-        <f>'Para Histograma'!T609</f>
         <v>0</v>
       </c>
       <c r="M33" s="1357">
-        <f>'Para Histograma'!U609</f>
         <v>0</v>
       </c>
       <c r="N33" s="1357">
-        <f>'Para Histograma'!V609</f>
         <v>1</v>
       </c>
       <c r="O33" s="1357">
-        <f>'Para Histograma'!W609</f>
         <v>1</v>
       </c>
       <c r="P33" s="1357">
-        <f>'Para Histograma'!X609</f>
         <v>0</v>
       </c>
       <c r="Q33" s="1357">
-        <f>'Para Histograma'!Y609</f>
         <v>0</v>
       </c>
       <c r="R33" s="1357">
-        <f>'Para Histograma'!Z609</f>
         <v>0</v>
       </c>
       <c r="S33" s="1357">
-        <f>'Para Histograma'!AA609</f>
         <v>0</v>
       </c>
       <c r="T33" s="1357">
-        <f>'Para Histograma'!AB609</f>
         <v>0</v>
       </c>
       <c r="U33" s="1357">
-        <f>'Para Histograma'!AC609</f>
         <v>0</v>
       </c>
     </row>
@@ -24476,7 +23762,6 @@
     </row>
     <row r="35" spans="2:21" s="1379" customFormat="1">
       <c r="B35" s="1500" t="str">
-        <f>'Para Histograma'!D610</f>
         <v>TERMOHIGÓMETRO</v>
       </c>
       <c r="C35" s="1356" t="inlineStr">
@@ -24485,75 +23770,57 @@
         </is>
       </c>
       <c r="D35" s="1357">
-        <f>'Para Histograma'!L610</f>
         <v>0</v>
       </c>
       <c r="E35" s="1357">
-        <f>'Para Histograma'!M610</f>
         <v>0</v>
       </c>
       <c r="F35" s="1357">
-        <f>'Para Histograma'!N610</f>
         <v>0</v>
       </c>
       <c r="G35" s="1357">
-        <f>'Para Histograma'!O610</f>
         <v>0</v>
       </c>
       <c r="H35" s="1357">
-        <f>'Para Histograma'!P610</f>
         <v>0</v>
       </c>
       <c r="I35" s="1357">
-        <f>'Para Histograma'!Q610</f>
         <v>0</v>
       </c>
       <c r="J35" s="1357">
-        <f>'Para Histograma'!R610</f>
         <v>0</v>
       </c>
       <c r="K35" s="1357">
-        <f>'Para Histograma'!S610</f>
         <v>0</v>
       </c>
       <c r="L35" s="1357">
-        <f>'Para Histograma'!T610</f>
         <v>0</v>
       </c>
       <c r="M35" s="1357">
-        <f>'Para Histograma'!U610</f>
         <v>0</v>
       </c>
       <c r="N35" s="1357">
-        <f>'Para Histograma'!V610</f>
         <v>1</v>
       </c>
       <c r="O35" s="1357">
-        <f>'Para Histograma'!W610</f>
         <v>1</v>
       </c>
       <c r="P35" s="1357">
-        <f>'Para Histograma'!X610</f>
         <v>0</v>
       </c>
       <c r="Q35" s="1357">
-        <f>'Para Histograma'!Y610</f>
         <v>0</v>
       </c>
       <c r="R35" s="1357">
-        <f>'Para Histograma'!Z610</f>
         <v>0</v>
       </c>
       <c r="S35" s="1357">
-        <f>'Para Histograma'!AA610</f>
         <v>0</v>
       </c>
       <c r="T35" s="1357">
-        <f>'Para Histograma'!AB610</f>
         <v>0</v>
       </c>
       <c r="U35" s="1357">
-        <f>'Para Histograma'!AC610</f>
         <v>0</v>
       </c>
     </row>
@@ -24585,7 +23852,6 @@
     </row>
     <row r="37" spans="2:21" s="1379" customFormat="1">
       <c r="B37" s="1500" t="str">
-        <f>'Para Histograma'!D611</f>
         <v>PIRÓMETRO</v>
       </c>
       <c r="C37" s="1356" t="inlineStr">
@@ -24594,75 +23860,57 @@
         </is>
       </c>
       <c r="D37" s="1357">
-        <f>'Para Histograma'!L611</f>
         <v>0</v>
       </c>
       <c r="E37" s="1357">
-        <f>'Para Histograma'!M611</f>
         <v>0</v>
       </c>
       <c r="F37" s="1357">
-        <f>'Para Histograma'!N611</f>
         <v>0</v>
       </c>
       <c r="G37" s="1357">
-        <f>'Para Histograma'!O611</f>
         <v>0</v>
       </c>
       <c r="H37" s="1357">
-        <f>'Para Histograma'!P611</f>
         <v>0</v>
       </c>
       <c r="I37" s="1357">
-        <f>'Para Histograma'!Q611</f>
         <v>0</v>
       </c>
       <c r="J37" s="1357">
-        <f>'Para Histograma'!R611</f>
         <v>0</v>
       </c>
       <c r="K37" s="1357">
-        <f>'Para Histograma'!S611</f>
         <v>0</v>
       </c>
       <c r="L37" s="1357">
-        <f>'Para Histograma'!T611</f>
         <v>0</v>
       </c>
       <c r="M37" s="1357">
-        <f>'Para Histograma'!U611</f>
         <v>0</v>
       </c>
       <c r="N37" s="1357">
-        <f>'Para Histograma'!V611</f>
         <v>1</v>
       </c>
       <c r="O37" s="1357">
-        <f>'Para Histograma'!W611</f>
         <v>1</v>
       </c>
       <c r="P37" s="1357">
-        <f>'Para Histograma'!X611</f>
         <v>0</v>
       </c>
       <c r="Q37" s="1357">
-        <f>'Para Histograma'!Y611</f>
         <v>0</v>
       </c>
       <c r="R37" s="1357">
-        <f>'Para Histograma'!Z611</f>
         <v>0</v>
       </c>
       <c r="S37" s="1357">
-        <f>'Para Histograma'!AA611</f>
         <v>0</v>
       </c>
       <c r="T37" s="1357">
-        <f>'Para Histograma'!AB611</f>
         <v>0</v>
       </c>
       <c r="U37" s="1357">
-        <f>'Para Histograma'!AC611</f>
         <v>0</v>
       </c>
     </row>
@@ -24694,7 +23942,6 @@
     </row>
     <row r="39" spans="2:21" s="1379" customFormat="1">
       <c r="B39" s="1500" t="str">
-        <f>'Para Histograma'!D612</f>
         <v>TALADRO PERCUTOR</v>
       </c>
       <c r="C39" s="1356" t="inlineStr">
@@ -24703,75 +23950,57 @@
         </is>
       </c>
       <c r="D39" s="1357">
-        <f>'Para Histograma'!L612</f>
         <v>0</v>
       </c>
       <c r="E39" s="1357">
-        <f>'Para Histograma'!M612</f>
         <v>0</v>
       </c>
       <c r="F39" s="1357">
-        <f>'Para Histograma'!N612</f>
         <v>0</v>
       </c>
       <c r="G39" s="1357">
-        <f>'Para Histograma'!O612</f>
         <v>0</v>
       </c>
       <c r="H39" s="1357">
-        <f>'Para Histograma'!P612</f>
         <v>0</v>
       </c>
       <c r="I39" s="1357">
-        <f>'Para Histograma'!Q612</f>
         <v>0</v>
       </c>
       <c r="J39" s="1357">
-        <f>'Para Histograma'!R612</f>
         <v>1</v>
       </c>
       <c r="K39" s="1357">
-        <f>'Para Histograma'!S612</f>
         <v>1</v>
       </c>
       <c r="L39" s="1357">
-        <f>'Para Histograma'!T612</f>
         <v>2</v>
       </c>
       <c r="M39" s="1357">
-        <f>'Para Histograma'!U612</f>
         <v>1</v>
       </c>
       <c r="N39" s="1357">
-        <f>'Para Histograma'!V612</f>
         <v>1</v>
       </c>
       <c r="O39" s="1357">
-        <f>'Para Histograma'!W612</f>
         <v>0</v>
       </c>
       <c r="P39" s="1357">
-        <f>'Para Histograma'!X612</f>
         <v>0</v>
       </c>
       <c r="Q39" s="1357">
-        <f>'Para Histograma'!Y612</f>
         <v>0</v>
       </c>
       <c r="R39" s="1357">
-        <f>'Para Histograma'!Z612</f>
         <v>0</v>
       </c>
       <c r="S39" s="1357">
-        <f>'Para Histograma'!AA612</f>
         <v>0</v>
       </c>
       <c r="T39" s="1357">
-        <f>'Para Histograma'!AB612</f>
         <v>0</v>
       </c>
       <c r="U39" s="1357">
-        <f>'Para Histograma'!AC612</f>
         <v>0</v>
       </c>
     </row>
@@ -24803,7 +24032,6 @@
     </row>
     <row r="41" spans="2:21" s="1379" customFormat="1">
       <c r="B41" s="1500" t="str">
-        <f>'Para Histograma'!D613</f>
         <v>MOTOBOMBA</v>
       </c>
       <c r="C41" s="1356" t="inlineStr">
@@ -24812,75 +24040,57 @@
         </is>
       </c>
       <c r="D41" s="1357">
-        <f>'Para Histograma'!L613</f>
         <v>0</v>
       </c>
       <c r="E41" s="1357">
-        <f>'Para Histograma'!M613</f>
         <v>0</v>
       </c>
       <c r="F41" s="1357">
-        <f>'Para Histograma'!N613</f>
         <v>0</v>
       </c>
       <c r="G41" s="1357">
-        <f>'Para Histograma'!O613</f>
         <v>0</v>
       </c>
       <c r="H41" s="1357">
-        <f>'Para Histograma'!P613</f>
         <v>0</v>
       </c>
       <c r="I41" s="1357">
-        <f>'Para Histograma'!Q613</f>
         <v>0</v>
       </c>
       <c r="J41" s="1357">
-        <f>'Para Histograma'!R613</f>
         <v>0</v>
       </c>
       <c r="K41" s="1357">
-        <f>'Para Histograma'!S613</f>
         <v>0</v>
       </c>
       <c r="L41" s="1357">
-        <f>'Para Histograma'!T613</f>
         <v>0</v>
       </c>
       <c r="M41" s="1357">
-        <f>'Para Histograma'!U613</f>
         <v>0</v>
       </c>
       <c r="N41" s="1357">
-        <f>'Para Histograma'!V613</f>
         <v>0</v>
       </c>
       <c r="O41" s="1357">
-        <f>'Para Histograma'!W613</f>
         <v>0</v>
       </c>
       <c r="P41" s="1357">
-        <f>'Para Histograma'!X613</f>
         <v>0</v>
       </c>
       <c r="Q41" s="1357">
-        <f>'Para Histograma'!Y613</f>
         <v>0</v>
       </c>
       <c r="R41" s="1357">
-        <f>'Para Histograma'!Z613</f>
         <v>0</v>
       </c>
       <c r="S41" s="1357">
-        <f>'Para Histograma'!AA613</f>
         <v>1</v>
       </c>
       <c r="T41" s="1357">
-        <f>'Para Histograma'!AB613</f>
         <v>0</v>
       </c>
       <c r="U41" s="1357">
-        <f>'Para Histograma'!AC613</f>
         <v>0</v>
       </c>
     </row>
@@ -24912,7 +24122,6 @@
     </row>
     <row r="43" spans="2:21" s="1379" customFormat="1">
       <c r="B43" s="1500" t="str">
-        <f>'Para Histograma'!D614</f>
         <v>BOMBA PARA PRUEBAS HIDROSTÁTICAS</v>
       </c>
       <c r="C43" s="1356" t="inlineStr">
@@ -24921,75 +24130,57 @@
         </is>
       </c>
       <c r="D43" s="1357">
-        <f>'Para Histograma'!L614</f>
         <v>0</v>
       </c>
       <c r="E43" s="1357">
-        <f>'Para Histograma'!M614</f>
         <v>0</v>
       </c>
       <c r="F43" s="1357">
-        <f>'Para Histograma'!N614</f>
         <v>0</v>
       </c>
       <c r="G43" s="1357">
-        <f>'Para Histograma'!O614</f>
         <v>0</v>
       </c>
       <c r="H43" s="1357">
-        <f>'Para Histograma'!P614</f>
         <v>0</v>
       </c>
       <c r="I43" s="1357">
-        <f>'Para Histograma'!Q614</f>
         <v>0</v>
       </c>
       <c r="J43" s="1357">
-        <f>'Para Histograma'!R614</f>
         <v>0</v>
       </c>
       <c r="K43" s="1357">
-        <f>'Para Histograma'!S614</f>
         <v>0</v>
       </c>
       <c r="L43" s="1357">
-        <f>'Para Histograma'!T614</f>
         <v>0</v>
       </c>
       <c r="M43" s="1357">
-        <f>'Para Histograma'!U614</f>
         <v>0</v>
       </c>
       <c r="N43" s="1357">
-        <f>'Para Histograma'!V614</f>
         <v>0</v>
       </c>
       <c r="O43" s="1357">
-        <f>'Para Histograma'!W614</f>
         <v>0</v>
       </c>
       <c r="P43" s="1357">
-        <f>'Para Histograma'!X614</f>
         <v>0</v>
       </c>
       <c r="Q43" s="1357">
-        <f>'Para Histograma'!Y614</f>
         <v>0</v>
       </c>
       <c r="R43" s="1357">
-        <f>'Para Histograma'!Z614</f>
         <v>0</v>
       </c>
       <c r="S43" s="1357">
-        <f>'Para Histograma'!AA614</f>
         <v>1</v>
       </c>
       <c r="T43" s="1357">
-        <f>'Para Histograma'!AB614</f>
         <v>0</v>
       </c>
       <c r="U43" s="1357">
-        <f>'Para Histograma'!AC614</f>
         <v>0</v>
       </c>
     </row>
@@ -25021,7 +24212,6 @@
     </row>
     <row r="45" spans="2:21" s="1379" customFormat="1">
       <c r="B45" s="1500" t="str">
-        <f>'Para Histograma'!D615</f>
         <v>TIRFOR</v>
       </c>
       <c r="C45" s="1356" t="inlineStr">
@@ -25030,75 +24220,57 @@
         </is>
       </c>
       <c r="D45" s="1357">
-        <f>'Para Histograma'!L615</f>
         <v>0</v>
       </c>
       <c r="E45" s="1357">
-        <f>'Para Histograma'!M615</f>
         <v>0</v>
       </c>
       <c r="F45" s="1357">
-        <f>'Para Histograma'!N615</f>
         <v>0</v>
       </c>
       <c r="G45" s="1357">
-        <f>'Para Histograma'!O615</f>
         <v>0</v>
       </c>
       <c r="H45" s="1357">
-        <f>'Para Histograma'!P615</f>
         <v>0</v>
       </c>
       <c r="I45" s="1357">
-        <f>'Para Histograma'!Q615</f>
         <v>0</v>
       </c>
       <c r="J45" s="1357">
-        <f>'Para Histograma'!R615</f>
         <v>0</v>
       </c>
       <c r="K45" s="1357">
-        <f>'Para Histograma'!S615</f>
         <v>0</v>
       </c>
       <c r="L45" s="1357">
-        <f>'Para Histograma'!T615</f>
         <v>0</v>
       </c>
       <c r="M45" s="1357">
-        <f>'Para Histograma'!U615</f>
         <v>1</v>
       </c>
       <c r="N45" s="1357">
-        <f>'Para Histograma'!V615</f>
         <v>1</v>
       </c>
       <c r="O45" s="1357">
-        <f>'Para Histograma'!W615</f>
         <v>0</v>
       </c>
       <c r="P45" s="1357">
-        <f>'Para Histograma'!X615</f>
         <v>0</v>
       </c>
       <c r="Q45" s="1357">
-        <f>'Para Histograma'!Y615</f>
         <v>0</v>
       </c>
       <c r="R45" s="1357">
-        <f>'Para Histograma'!Z615</f>
         <v>0</v>
       </c>
       <c r="S45" s="1357">
-        <f>'Para Histograma'!AA615</f>
         <v>0</v>
       </c>
       <c r="T45" s="1357">
-        <f>'Para Histograma'!AB615</f>
         <v>0</v>
       </c>
       <c r="U45" s="1357">
-        <f>'Para Histograma'!AC615</f>
         <v>0</v>
       </c>
     </row>
@@ -25130,7 +24302,6 @@
     </row>
     <row r="47" spans="2:21" s="1379" customFormat="1">
       <c r="B47" s="1500" t="str">
-        <f>'Para Histograma'!D616</f>
         <v>ESMERIL ANGULAR</v>
       </c>
       <c r="C47" s="1356" t="inlineStr">
@@ -25139,75 +24310,57 @@
         </is>
       </c>
       <c r="D47" s="1357">
-        <f>'Para Histograma'!L616</f>
         <v>0</v>
       </c>
       <c r="E47" s="1357">
-        <f>'Para Histograma'!M616</f>
         <v>0</v>
       </c>
       <c r="F47" s="1357">
-        <f>'Para Histograma'!N616</f>
         <v>0</v>
       </c>
       <c r="G47" s="1357">
-        <f>'Para Histograma'!O616</f>
         <v>0</v>
       </c>
       <c r="H47" s="1357">
-        <f>'Para Histograma'!P616</f>
         <v>0</v>
       </c>
       <c r="I47" s="1357">
-        <f>'Para Histograma'!Q616</f>
         <v>0</v>
       </c>
       <c r="J47" s="1357">
-        <f>'Para Histograma'!R616</f>
         <v>0</v>
       </c>
       <c r="K47" s="1357">
-        <f>'Para Histograma'!S616</f>
         <v>2</v>
       </c>
       <c r="L47" s="1357">
-        <f>'Para Histograma'!T616</f>
         <v>2</v>
       </c>
       <c r="M47" s="1357">
-        <f>'Para Histograma'!U616</f>
         <v>2</v>
       </c>
       <c r="N47" s="1357">
-        <f>'Para Histograma'!V616</f>
         <v>2</v>
       </c>
       <c r="O47" s="1357">
-        <f>'Para Histograma'!W616</f>
         <v>2</v>
       </c>
       <c r="P47" s="1357">
-        <f>'Para Histograma'!X616</f>
         <v>2</v>
       </c>
       <c r="Q47" s="1357">
-        <f>'Para Histograma'!Y616</f>
         <v>2</v>
       </c>
       <c r="R47" s="1357">
-        <f>'Para Histograma'!Z616</f>
         <v>1</v>
       </c>
       <c r="S47" s="1357">
-        <f>'Para Histograma'!AA616</f>
         <v>1</v>
       </c>
       <c r="T47" s="1357">
-        <f>'Para Histograma'!AB616</f>
         <v>1</v>
       </c>
       <c r="U47" s="1357">
-        <f>'Para Histograma'!AC616</f>
         <v>0</v>
       </c>
     </row>
@@ -25239,7 +24392,6 @@
     </row>
     <row r="49" spans="2:21" s="1379" customFormat="1">
       <c r="B49" s="1500" t="str">
-        <f>'Para Histograma'!D617</f>
         <v>ANDAMIOS</v>
       </c>
       <c r="C49" s="1356" t="inlineStr">
@@ -25248,75 +24400,57 @@
         </is>
       </c>
       <c r="D49" s="1357">
-        <f>'Para Histograma'!L617</f>
         <v>0</v>
       </c>
       <c r="E49" s="1357">
-        <f>'Para Histograma'!M617</f>
         <v>0</v>
       </c>
       <c r="F49" s="1357">
-        <f>'Para Histograma'!N617</f>
         <v>0</v>
       </c>
       <c r="G49" s="1357">
-        <f>'Para Histograma'!O617</f>
         <v>0</v>
       </c>
       <c r="H49" s="1357">
-        <f>'Para Histograma'!P617</f>
         <v>0</v>
       </c>
       <c r="I49" s="1357">
-        <f>'Para Histograma'!Q617</f>
         <v>0</v>
       </c>
       <c r="J49" s="1357">
-        <f>'Para Histograma'!R617</f>
         <v>0</v>
       </c>
       <c r="K49" s="1357">
-        <f>'Para Histograma'!S617</f>
         <v>6</v>
       </c>
       <c r="L49" s="1357">
-        <f>'Para Histograma'!T617</f>
         <v>6</v>
       </c>
       <c r="M49" s="1357">
-        <f>'Para Histograma'!U617</f>
         <v>6</v>
       </c>
       <c r="N49" s="1357">
-        <f>'Para Histograma'!V617</f>
         <v>6</v>
       </c>
       <c r="O49" s="1357">
-        <f>'Para Histograma'!W617</f>
         <v>7</v>
       </c>
       <c r="P49" s="1357">
-        <f>'Para Histograma'!X617</f>
         <v>6</v>
       </c>
       <c r="Q49" s="1357">
-        <f>'Para Histograma'!Y617</f>
         <v>6</v>
       </c>
       <c r="R49" s="1357">
-        <f>'Para Histograma'!Z617</f>
         <v>3</v>
       </c>
       <c r="S49" s="1357">
-        <f>'Para Histograma'!AA617</f>
         <v>3</v>
       </c>
       <c r="T49" s="1357">
-        <f>'Para Histograma'!AB617</f>
         <v>0</v>
       </c>
       <c r="U49" s="1357">
-        <f>'Para Histograma'!AC617</f>
         <v>0</v>
       </c>
     </row>
@@ -25348,7 +24482,6 @@
     </row>
     <row r="51" spans="2:21" s="1379" customFormat="1">
       <c r="B51" s="1500" t="str">
-        <f>'Para Histograma'!D618</f>
         <v>TALADRO</v>
       </c>
       <c r="C51" s="1356" t="inlineStr">
@@ -25357,75 +24490,57 @@
         </is>
       </c>
       <c r="D51" s="1357">
-        <f>'Para Histograma'!L618</f>
         <v>0</v>
       </c>
       <c r="E51" s="1357">
-        <f>'Para Histograma'!M618</f>
         <v>0</v>
       </c>
       <c r="F51" s="1357">
-        <f>'Para Histograma'!N618</f>
         <v>0</v>
       </c>
       <c r="G51" s="1357">
-        <f>'Para Histograma'!O618</f>
         <v>0</v>
       </c>
       <c r="H51" s="1357">
-        <f>'Para Histograma'!P618</f>
         <v>0</v>
       </c>
       <c r="I51" s="1357">
-        <f>'Para Histograma'!Q618</f>
         <v>0</v>
       </c>
       <c r="J51" s="1357">
-        <f>'Para Histograma'!R618</f>
         <v>0</v>
       </c>
       <c r="K51" s="1357">
-        <f>'Para Histograma'!S618</f>
         <v>1</v>
       </c>
       <c r="L51" s="1357">
-        <f>'Para Histograma'!T618</f>
         <v>0</v>
       </c>
       <c r="M51" s="1357">
-        <f>'Para Histograma'!U618</f>
         <v>0</v>
       </c>
       <c r="N51" s="1357">
-        <f>'Para Histograma'!V618</f>
         <v>0</v>
       </c>
       <c r="O51" s="1357">
-        <f>'Para Histograma'!W618</f>
         <v>0</v>
       </c>
       <c r="P51" s="1357">
-        <f>'Para Histograma'!X618</f>
         <v>0</v>
       </c>
       <c r="Q51" s="1357">
-        <f>'Para Histograma'!Y618</f>
         <v>0</v>
       </c>
       <c r="R51" s="1357">
-        <f>'Para Histograma'!Z618</f>
         <v>0</v>
       </c>
       <c r="S51" s="1357">
-        <f>'Para Histograma'!AA618</f>
         <v>0</v>
       </c>
       <c r="T51" s="1357">
-        <f>'Para Histograma'!AB618</f>
         <v>0</v>
       </c>
       <c r="U51" s="1357">
-        <f>'Para Histograma'!AC618</f>
         <v>0</v>
       </c>
     </row>
@@ -25457,7 +24572,6 @@
     </row>
     <row r="53" spans="2:21" s="1379" customFormat="1">
       <c r="B53" s="1500" t="str">
-        <f>'Para Histograma'!D619</f>
         <v>MULTIMETRO</v>
       </c>
       <c r="C53" s="1356" t="inlineStr">
@@ -25466,75 +24580,57 @@
         </is>
       </c>
       <c r="D53" s="1357">
-        <f>'Para Histograma'!L619</f>
         <v>0</v>
       </c>
       <c r="E53" s="1357">
-        <f>'Para Histograma'!M619</f>
         <v>0</v>
       </c>
       <c r="F53" s="1357">
-        <f>'Para Histograma'!N619</f>
         <v>0</v>
       </c>
       <c r="G53" s="1357">
-        <f>'Para Histograma'!O619</f>
         <v>0</v>
       </c>
       <c r="H53" s="1357">
-        <f>'Para Histograma'!P619</f>
         <v>0</v>
       </c>
       <c r="I53" s="1357">
-        <f>'Para Histograma'!Q619</f>
         <v>0</v>
       </c>
       <c r="J53" s="1357">
-        <f>'Para Histograma'!R619</f>
         <v>1</v>
       </c>
       <c r="K53" s="1357">
-        <f>'Para Histograma'!S619</f>
         <v>1</v>
       </c>
       <c r="L53" s="1357">
-        <f>'Para Histograma'!T619</f>
         <v>1</v>
       </c>
       <c r="M53" s="1357">
-        <f>'Para Histograma'!U619</f>
         <v>1</v>
       </c>
       <c r="N53" s="1357">
-        <f>'Para Histograma'!V619</f>
         <v>1</v>
       </c>
       <c r="O53" s="1357">
-        <f>'Para Histograma'!W619</f>
         <v>1</v>
       </c>
       <c r="P53" s="1357">
-        <f>'Para Histograma'!X619</f>
         <v>0</v>
       </c>
       <c r="Q53" s="1357">
-        <f>'Para Histograma'!Y619</f>
         <v>0</v>
       </c>
       <c r="R53" s="1357">
-        <f>'Para Histograma'!Z619</f>
         <v>0</v>
       </c>
       <c r="S53" s="1357">
-        <f>'Para Histograma'!AA619</f>
         <v>0</v>
       </c>
       <c r="T53" s="1357">
-        <f>'Para Histograma'!AB619</f>
         <v>0</v>
       </c>
       <c r="U53" s="1357">
-        <f>'Para Histograma'!AC619</f>
         <v>0</v>
       </c>
     </row>
@@ -25566,7 +24662,6 @@
     </row>
     <row r="55" spans="2:21" s="1379" customFormat="1">
       <c r="B55" s="1500" t="str">
-        <f>'Para Histograma'!D620</f>
         <v>MEGÓMETRO</v>
       </c>
       <c r="C55" s="1356" t="inlineStr">
@@ -25575,75 +24670,57 @@
         </is>
       </c>
       <c r="D55" s="1357">
-        <f>'Para Histograma'!L620</f>
         <v>0</v>
       </c>
       <c r="E55" s="1357">
-        <f>'Para Histograma'!M620</f>
         <v>0</v>
       </c>
       <c r="F55" s="1357">
-        <f>'Para Histograma'!N620</f>
         <v>0</v>
       </c>
       <c r="G55" s="1357">
-        <f>'Para Histograma'!O620</f>
         <v>0</v>
       </c>
       <c r="H55" s="1357">
-        <f>'Para Histograma'!P620</f>
         <v>0</v>
       </c>
       <c r="I55" s="1357">
-        <f>'Para Histograma'!Q620</f>
         <v>0</v>
       </c>
       <c r="J55" s="1357">
-        <f>'Para Histograma'!R620</f>
         <v>0</v>
       </c>
       <c r="K55" s="1357">
-        <f>'Para Histograma'!S620</f>
         <v>1</v>
       </c>
       <c r="L55" s="1357">
-        <f>'Para Histograma'!T620</f>
         <v>0</v>
       </c>
       <c r="M55" s="1357">
-        <f>'Para Histograma'!U620</f>
         <v>0</v>
       </c>
       <c r="N55" s="1357">
-        <f>'Para Histograma'!V620</f>
         <v>0</v>
       </c>
       <c r="O55" s="1357">
-        <f>'Para Histograma'!W620</f>
         <v>0</v>
       </c>
       <c r="P55" s="1357">
-        <f>'Para Histograma'!X620</f>
         <v>0</v>
       </c>
       <c r="Q55" s="1357">
-        <f>'Para Histograma'!Y620</f>
         <v>0</v>
       </c>
       <c r="R55" s="1357">
-        <f>'Para Histograma'!Z620</f>
         <v>0</v>
       </c>
       <c r="S55" s="1357">
-        <f>'Para Histograma'!AA620</f>
         <v>0</v>
       </c>
       <c r="T55" s="1357">
-        <f>'Para Histograma'!AB620</f>
         <v>0</v>
       </c>
       <c r="U55" s="1357">
-        <f>'Para Histograma'!AC620</f>
         <v>0</v>
       </c>
     </row>
@@ -25675,7 +24752,6 @@
     </row>
     <row r="57" spans="2:21" s="1379" customFormat="1">
       <c r="B57" s="1500" t="str">
-        <f>'Para Histograma'!D621</f>
         <v>MEGOMETRO</v>
       </c>
       <c r="C57" s="1356" t="inlineStr">
@@ -25684,75 +24760,57 @@
         </is>
       </c>
       <c r="D57" s="1357">
-        <f>'Para Histograma'!L621</f>
         <v>0</v>
       </c>
       <c r="E57" s="1357">
-        <f>'Para Histograma'!M621</f>
         <v>0</v>
       </c>
       <c r="F57" s="1357">
-        <f>'Para Histograma'!N621</f>
         <v>0</v>
       </c>
       <c r="G57" s="1357">
-        <f>'Para Histograma'!O621</f>
         <v>0</v>
       </c>
       <c r="H57" s="1357">
-        <f>'Para Histograma'!P621</f>
         <v>0</v>
       </c>
       <c r="I57" s="1357">
-        <f>'Para Histograma'!Q621</f>
         <v>0</v>
       </c>
       <c r="J57" s="1357">
-        <f>'Para Histograma'!R621</f>
         <v>1</v>
       </c>
       <c r="K57" s="1357">
-        <f>'Para Histograma'!S621</f>
         <v>1</v>
       </c>
       <c r="L57" s="1357">
-        <f>'Para Histograma'!T621</f>
         <v>1</v>
       </c>
       <c r="M57" s="1357">
-        <f>'Para Histograma'!U621</f>
         <v>1</v>
       </c>
       <c r="N57" s="1357">
-        <f>'Para Histograma'!V621</f>
         <v>1</v>
       </c>
       <c r="O57" s="1357">
-        <f>'Para Histograma'!W621</f>
         <v>0</v>
       </c>
       <c r="P57" s="1357">
-        <f>'Para Histograma'!X621</f>
         <v>0</v>
       </c>
       <c r="Q57" s="1357">
-        <f>'Para Histograma'!Y621</f>
         <v>0</v>
       </c>
       <c r="R57" s="1357">
-        <f>'Para Histograma'!Z621</f>
         <v>0</v>
       </c>
       <c r="S57" s="1357">
-        <f>'Para Histograma'!AA621</f>
         <v>0</v>
       </c>
       <c r="T57" s="1357">
-        <f>'Para Histograma'!AB621</f>
         <v>0</v>
       </c>
       <c r="U57" s="1357">
-        <f>'Para Histograma'!AC621</f>
         <v>0</v>
       </c>
     </row>
@@ -25784,7 +24842,6 @@
     </row>
     <row r="59" spans="2:21" s="1379" customFormat="1">
       <c r="B59" s="1500" t="str">
-        <f>'Para Histograma'!D622</f>
         <v>GENERADOR DE TONO</v>
       </c>
       <c r="C59" s="1356" t="inlineStr">
@@ -25793,75 +24850,57 @@
         </is>
       </c>
       <c r="D59" s="1357">
-        <f>'Para Histograma'!L622</f>
         <v>0</v>
       </c>
       <c r="E59" s="1357">
-        <f>'Para Histograma'!M622</f>
         <v>0</v>
       </c>
       <c r="F59" s="1357">
-        <f>'Para Histograma'!N622</f>
         <v>0</v>
       </c>
       <c r="G59" s="1357">
-        <f>'Para Histograma'!O622</f>
         <v>0</v>
       </c>
       <c r="H59" s="1357">
-        <f>'Para Histograma'!P622</f>
         <v>0</v>
       </c>
       <c r="I59" s="1357">
-        <f>'Para Histograma'!Q622</f>
         <v>0</v>
       </c>
       <c r="J59" s="1357">
-        <f>'Para Histograma'!R622</f>
         <v>1</v>
       </c>
       <c r="K59" s="1357">
-        <f>'Para Histograma'!S622</f>
         <v>0</v>
       </c>
       <c r="L59" s="1357">
-        <f>'Para Histograma'!T622</f>
         <v>0</v>
       </c>
       <c r="M59" s="1357">
-        <f>'Para Histograma'!U622</f>
         <v>0</v>
       </c>
       <c r="N59" s="1357">
-        <f>'Para Histograma'!V622</f>
         <v>0</v>
       </c>
       <c r="O59" s="1357">
-        <f>'Para Histograma'!W622</f>
         <v>0</v>
       </c>
       <c r="P59" s="1357">
-        <f>'Para Histograma'!X622</f>
         <v>0</v>
       </c>
       <c r="Q59" s="1357">
-        <f>'Para Histograma'!Y622</f>
         <v>0</v>
       </c>
       <c r="R59" s="1357">
-        <f>'Para Histograma'!Z622</f>
         <v>0</v>
       </c>
       <c r="S59" s="1357">
-        <f>'Para Histograma'!AA622</f>
         <v>0</v>
       </c>
       <c r="T59" s="1357">
-        <f>'Para Histograma'!AB622</f>
         <v>0</v>
       </c>
       <c r="U59" s="1357">
-        <f>'Para Histograma'!AC622</f>
         <v>0</v>
       </c>
     </row>
@@ -25893,7 +24932,6 @@
     </row>
     <row r="61" spans="2:21" s="1379" customFormat="1">
       <c r="B61" s="1500" t="str">
-        <f>'Para Histograma'!D623</f>
         <v>DOBLADORA</v>
       </c>
       <c r="C61" s="1356" t="inlineStr">
@@ -25902,75 +24940,57 @@
         </is>
       </c>
       <c r="D61" s="1357">
-        <f>'Para Histograma'!L623</f>
         <v>0</v>
       </c>
       <c r="E61" s="1357">
-        <f>'Para Histograma'!M623</f>
         <v>0</v>
       </c>
       <c r="F61" s="1357">
-        <f>'Para Histograma'!N623</f>
         <v>0</v>
       </c>
       <c r="G61" s="1357">
-        <f>'Para Histograma'!O623</f>
         <v>0</v>
       </c>
       <c r="H61" s="1357">
-        <f>'Para Histograma'!P623</f>
         <v>0</v>
       </c>
       <c r="I61" s="1357">
-        <f>'Para Histograma'!Q623</f>
         <v>0</v>
       </c>
       <c r="J61" s="1357">
-        <f>'Para Histograma'!R623</f>
         <v>0</v>
       </c>
       <c r="K61" s="1357">
-        <f>'Para Histograma'!S623</f>
         <v>0</v>
       </c>
       <c r="L61" s="1357">
-        <f>'Para Histograma'!T623</f>
         <v>0</v>
       </c>
       <c r="M61" s="1357">
-        <f>'Para Histograma'!U623</f>
         <v>0</v>
       </c>
       <c r="N61" s="1357">
-        <f>'Para Histograma'!V623</f>
         <v>0</v>
       </c>
       <c r="O61" s="1357">
-        <f>'Para Histograma'!W623</f>
         <v>0</v>
       </c>
       <c r="P61" s="1357">
-        <f>'Para Histograma'!X623</f>
         <v>0</v>
       </c>
       <c r="Q61" s="1357">
-        <f>'Para Histograma'!Y623</f>
         <v>0</v>
       </c>
       <c r="R61" s="1357">
-        <f>'Para Histograma'!Z623</f>
         <v>0</v>
       </c>
       <c r="S61" s="1357">
-        <f>'Para Histograma'!AA623</f>
         <v>1</v>
       </c>
       <c r="T61" s="1357">
-        <f>'Para Histograma'!AB623</f>
         <v>0</v>
       </c>
       <c r="U61" s="1357">
-        <f>'Para Histograma'!AC623</f>
         <v>0</v>
       </c>
     </row>
@@ -26034,75 +25054,57 @@
         </is>
       </c>
       <c r="D64" s="1361">
-        <f>SUMIF($C13:$C62,"Plan",D13:D62)</f>
         <v>0</v>
       </c>
       <c r="E64" s="1361">
-        <f t="shared" ref="E64:U64" si="0">SUMIF($C13:$C62,"Plan",E13:E62)</f>
         <v>0</v>
       </c>
       <c r="F64" s="1361">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G64" s="1361">
-        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="H64" s="1361">
-        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="I64" s="1361">
-        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="J64" s="1361">
-        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="K64" s="1361">
-        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="L64" s="1361">
-        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="M64" s="1361">
-        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="N64" s="1361">
-        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="O64" s="1361">
-        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="P64" s="1361">
-        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="Q64" s="1361">
-        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="R64" s="1361">
-        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="S64" s="1361">
-        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="T64" s="1361">
-        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="U64" s="1361">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -26114,75 +25116,57 @@
         </is>
       </c>
       <c r="D65" s="1493">
-        <f>SUMIF($C13:$C62,"Act.",D13:D62)</f>
         <v>0</v>
       </c>
       <c r="E65" s="1493">
-        <f t="shared" ref="E65:U65" si="1">SUMIF($C13:$C62,"Act.",E13:E62)</f>
         <v>0</v>
       </c>
       <c r="F65" s="1493">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="G65" s="1493">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="H65" s="1493">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I65" s="1493">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J65" s="1493">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K65" s="1493">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="L65" s="1493">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M65" s="1493">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N65" s="1493">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O65" s="1493">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="P65" s="1493">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Q65" s="1493">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R65" s="1493">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="S65" s="1493">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="T65" s="1493">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="U65" s="1493">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>